<commit_message>
results: refresh paper figure workbook + A1/A2 appendix charts (vintage 202607091035)
Re-ran paper_figure_data.R over the regenerated 2030 outputs; rebuilt
the paper-exhibit workbook (12 sheets) and re-pulled the FRED-sourced
A1 (GDP growth) and A2 (labor share) appendix charts from live data.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/figures/2030/paper_figure_data_2030.xlsx
+++ b/results/figures/2030/paper_figure_data_2030.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="238">
   <si>
     <t xml:space="preserve">AI-Fiscal — paper exhibits (FY 2030)</t>
   </si>
   <si>
-    <t xml:space="preserve">June 2026</t>
+    <t xml:space="preserve">July 2026</t>
   </si>
   <si>
     <t xml:space="preserve">The Budget Lab at Yale</t>
@@ -155,7 +155,7 @@
     <t xml:space="preserve">Debt-to-GDP by scenario (BLSMM)</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: Slow / Moderate / Rapid AI-adoption variants; Karger et al. 2026, CBO 2025, TBL calculations.</t>
+    <t xml:space="preserve">Notes: Slow / Moderate / Rapid AI-adoption variants; Karger et al. 2026, CBO February 2026, TBL calculations.</t>
   </si>
   <si>
     <t xml:space="preserve">Source: The Budget Lab at Yale AI-Fiscal microsimulation model, FY 2030.</t>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">0.033</t>
   </si>
   <si>
-    <t xml:space="preserve">2030 capital share (s_1)</t>
+    <t xml:space="preserve">2030 capital share (theta_1_K)</t>
   </si>
   <si>
     <t xml:space="preserve">0.45</t>
@@ -218,7 +218,7 @@
     <t xml:space="preserve">0.487</t>
   </si>
   <si>
-    <t xml:space="preserve">2030 labor share (1 - s_1)</t>
+    <t xml:space="preserve">2030 labor share (theta_1_L)</t>
   </si>
   <si>
     <t xml:space="preserve">0.55</t>
@@ -272,10 +272,10 @@
     <t xml:space="preserve">-0.00943271239531995</t>
   </si>
   <si>
-    <t xml:space="preserve">Labor-income inequality parameter (sigma)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sigma = 1 ± k · g_y on log(YiL);   k = 1.000</t>
+    <t xml:space="preserve">Labor-income inequality parameter (lambda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lambda = 1 ± k · g_y on log(y_l);   k = 1.000</t>
   </si>
   <si>
     <t xml:space="preserve">Compressive</t>
@@ -314,10 +314,10 @@
     <t xml:space="preserve">Baseline labor share (2025): 55.5%. Source: Karger, Buehler, Cox, Saint-Jacques, and Bjorkegren (2026), CBO (2026), and TBL Calculations.</t>
   </si>
   <si>
-    <t xml:space="preserve">Share mode shown: Reallocate (R). The Karger labor-share decline is imposed. Fixed-share (F) twins live in the share_mode_comparison sheet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Negative labor growth occurs when the labor share falls fast enough to outweigh productivity gains over the horizon. Aggregate labor income levels remain positive - see L0_B / L1_B in cell_params.</t>
+    <t xml:space="preserve">Share mode shown: Reallocate (R). The Karger labor-share decline is imposed; fixed-share (F) twins are reported separately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Negative labor growth occurs when the labor share falls fast enough to outweigh productivity gains over the horizon. Aggregate labor income levels remain positive - see y0_l_B / y1_l_B in cell_params.</t>
   </si>
   <si>
     <t xml:space="preserve">Subtitle: Change in federal revenue, including corporate tax wedge, FY 2030, Billions USD</t>
@@ -530,7 +530,7 @@
     <t xml:space="preserve">Notes: Real GDP from FRED GDPC1 (Bil. Chn. 2017$). 5-yr annualized log growth; projection extends GDP with the CBO baseline path. Reference lines = AI scenario GDP CAGRs.</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: BEA/BLS via FRED (GDPC1), CBO 2025 baseline, NBER recessions; The Budget Lab at Yale.</t>
+    <t xml:space="preserve">Source: BEA/BLS via FRED (GDPC1), CBO February 2026 baseline, NBER recessions; The Budget Lab at Yale.</t>
   </si>
   <si>
     <t xml:space="preserve">Year</t>
@@ -596,43 +596,148 @@
     <t xml:space="preserve">Notes: Per-scenario 2030 debt/GDP from the Budget Lab Small Macro Model (BLSMM).</t>
   </si>
   <si>
-    <t xml:space="preserve">r_ai_annual_target</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_rev_to_gdp_cbo_pp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prod_bump_pp_per_yr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_gstar_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_annualized_growth_horizon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_year_real_growth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_rgfr_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_rgfop_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_debt_year_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_gdp_nominal_year_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">blsmm_debt_to_gdp_year_pct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_debt_to_gdp_vs_baseline_pp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline</t>
+    <t xml:space="preserve">Scenario.ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI.Adoption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share.Mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share.Mode.(label)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labor.Scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI.GDP.CAGR.Target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ.Revenue-to-GDP.vs.CBO.(pp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Productivity.Bump.(pp/yr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GDP.Growth.g*.(%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annualized.Growth.(2025–Year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real.GDP.Growth.(Year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Federal.Revenue.Path.rgfr*.(%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rgfop*.(%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debt.($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nominal.GDP.($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debt-to-GDP.(%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ.Debt-to-GDP.vs.Baseline.(pp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blsmm_baseline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_M_F_S0_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_M_F_S2_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_M_F_S3_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_M_R_S0_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reallocate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_M_R_S2_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_M_R_S3_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_R_F_S0_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_R_F_S2_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_R_F_S3_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_R_R_S0_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_R_R_S2_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_R_R_S3_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_S_F_S0_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_S_F_S2_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_S_F_S3_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_S_R_S0_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_S_R_S2_V1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ai_S_R_S3_V1</t>
   </si>
 </sst>
 </file>
@@ -4690,19 +4795,26 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="46.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="20.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="25.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="21.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="22.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="33.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="24.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="21.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="22.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="19.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="26.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="28.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="34.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="12.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="20.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="9.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="13.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="20.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="30.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="27.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="19.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="31.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="24.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="32.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="12.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="11.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="18.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="17.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="32.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4722,22 +4834,22 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>99</v>
+        <v>190</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>194</v>
+        <v>115</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>195</v>
@@ -4760,781 +4872,1187 @@
       <c r="M6" s="3" t="s">
         <v>201</v>
       </c>
+      <c r="N6" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="R6" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B7"/>
-      <c r="C7" t="n">
+      <c r="C7"/>
+      <c r="D7"/>
+      <c r="E7"/>
+      <c r="F7"/>
+      <c r="G7"/>
+      <c r="H7"/>
+      <c r="I7"/>
+      <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="D7" t="n">
+      <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="E7" t="n">
+      <c r="L7" t="n">
         <v>2.05628646645455</v>
       </c>
-      <c r="F7" t="n">
+      <c r="M7" t="n">
         <v>0.0192829240109289</v>
       </c>
-      <c r="G7" t="n">
+      <c r="N7" t="n">
         <v>0.0181200848684659</v>
       </c>
-      <c r="H7" t="n">
+      <c r="O7" t="n">
         <v>17.6430302673608</v>
       </c>
-      <c r="I7" t="n">
+      <c r="P7" t="n">
         <v>19.7002691264359</v>
       </c>
-      <c r="J7" t="n">
+      <c r="Q7" t="n">
         <v>40202.2691888061</v>
       </c>
-      <c r="K7" t="n">
+      <c r="R7" t="n">
         <v>37445.0828604847</v>
       </c>
-      <c r="L7" t="n">
+      <c r="S7" t="n">
         <v>107.36328008298</v>
       </c>
-      <c r="M7" t="n">
+      <c r="T7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>144</v>
-      </c>
-      <c r="B8" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="C8" t="n">
+        <v>210</v>
+      </c>
+      <c r="B8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>212</v>
+      </c>
+      <c r="E8" t="s">
+        <v>213</v>
+      </c>
+      <c r="F8" t="s">
+        <v>214</v>
+      </c>
+      <c r="G8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H8" t="s">
+        <v>215</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="J8" t="n">
         <v>-0.148558309057403</v>
       </c>
-      <c r="D8" t="n">
+      <c r="K8" t="n">
         <v>0.683660008499217</v>
       </c>
-      <c r="E8" t="n">
+      <c r="L8" t="n">
         <v>2.74322307232682</v>
       </c>
-      <c r="F8" t="n">
+      <c r="M8" t="n">
         <v>0.0259999999925518</v>
       </c>
-      <c r="G8" t="n">
+      <c r="N8" t="n">
         <v>0.0251915636891986</v>
       </c>
-      <c r="H8" t="n">
+      <c r="O8" t="n">
         <v>17.4944719583034</v>
       </c>
-      <c r="I8" t="n">
+      <c r="P8" t="n">
         <v>19.0740365586506</v>
       </c>
-      <c r="J8" t="n">
+      <c r="Q8" t="n">
         <v>39889.4428134478</v>
       </c>
-      <c r="K8" t="n">
+      <c r="R8" t="n">
         <v>38666.9803218121</v>
       </c>
-      <c r="L8" t="n">
+      <c r="S8" t="n">
         <v>103.161515281156</v>
       </c>
-      <c r="M8" t="n">
+      <c r="T8" t="n">
         <v>-4.20176480182364</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="C9" t="n">
+        <v>216</v>
+      </c>
+      <c r="B9" t="s">
+        <v>211</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" t="s">
+        <v>212</v>
+      </c>
+      <c r="E9" t="s">
+        <v>213</v>
+      </c>
+      <c r="F9" t="s">
+        <v>217</v>
+      </c>
+      <c r="G9" t="s">
+        <v>84</v>
+      </c>
+      <c r="H9" t="s">
+        <v>215</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="J9" t="n">
         <v>-0.201752970943184</v>
       </c>
-      <c r="D9" t="n">
+      <c r="K9" t="n">
         <v>0.682857390632746</v>
       </c>
-      <c r="E9" t="n">
+      <c r="L9" t="n">
         <v>2.74241660773014</v>
       </c>
-      <c r="F9" t="n">
+      <c r="M9" t="n">
         <v>0.0259999999790508</v>
       </c>
-      <c r="G9" t="n">
+      <c r="N9" t="n">
         <v>0.025167981776919</v>
       </c>
-      <c r="H9" t="n">
+      <c r="O9" t="n">
         <v>17.4412772964176</v>
       </c>
-      <c r="I9" t="n">
+      <c r="P9" t="n">
         <v>19.0747717566163</v>
       </c>
-      <c r="J9" t="n">
+      <c r="Q9" t="n">
         <v>39956.2480542827</v>
       </c>
-      <c r="K9" t="n">
+      <c r="R9" t="n">
         <v>38670.5898664454</v>
       </c>
-      <c r="L9" t="n">
+      <c r="S9" t="n">
         <v>103.324640747083</v>
       </c>
-      <c r="M9" t="n">
+      <c r="T9" t="n">
         <v>-4.03863933589642</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>146</v>
-      </c>
-      <c r="B10" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="C10" t="n">
+        <v>218</v>
+      </c>
+      <c r="B10" t="s">
+        <v>211</v>
+      </c>
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" t="s">
+        <v>212</v>
+      </c>
+      <c r="E10" t="s">
+        <v>213</v>
+      </c>
+      <c r="F10" t="s">
+        <v>219</v>
+      </c>
+      <c r="G10" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" t="s">
+        <v>215</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="J10" t="n">
         <v>-0.0913881282996021</v>
       </c>
-      <c r="D10" t="n">
+      <c r="K10" t="n">
         <v>0.684522650605378</v>
       </c>
-      <c r="E10" t="n">
+      <c r="L10" t="n">
         <v>2.74408984884307</v>
       </c>
-      <c r="F10" t="n">
+      <c r="M10" t="n">
         <v>0.026000000008817</v>
       </c>
-      <c r="G10" t="n">
+      <c r="N10" t="n">
         <v>0.0252169107027416</v>
       </c>
-      <c r="H10" t="n">
+      <c r="O10" t="n">
         <v>17.5516421390612</v>
       </c>
-      <c r="I10" t="n">
+      <c r="P10" t="n">
         <v>19.0732463784814</v>
       </c>
-      <c r="J10" t="n">
+      <c r="Q10" t="n">
         <v>39817.6577279583</v>
       </c>
-      <c r="K10" t="n">
+      <c r="R10" t="n">
         <v>38663.1012949494</v>
       </c>
-      <c r="L10" t="n">
+      <c r="S10" t="n">
         <v>102.986197160443</v>
       </c>
-      <c r="M10" t="n">
+      <c r="T10" t="n">
         <v>-4.3770829225371</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>104</v>
-      </c>
-      <c r="B11" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="C11" t="n">
+        <v>220</v>
+      </c>
+      <c r="B11" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" t="s">
+        <v>221</v>
+      </c>
+      <c r="E11" t="s">
+        <v>222</v>
+      </c>
+      <c r="F11" t="s">
+        <v>214</v>
+      </c>
+      <c r="G11" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" t="s">
+        <v>215</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="J11" t="n">
         <v>-0.341006535077831</v>
       </c>
-      <c r="D11" t="n">
+      <c r="K11" t="n">
         <v>0.680756477697625</v>
       </c>
-      <c r="E11" t="n">
+      <c r="L11" t="n">
         <v>2.74030562568799</v>
       </c>
-      <c r="F11" t="n">
+      <c r="M11" t="n">
         <v>0.0259999999844491</v>
       </c>
-      <c r="G11" t="n">
+      <c r="N11" t="n">
         <v>0.0251062596763245</v>
       </c>
-      <c r="H11" t="n">
+      <c r="O11" t="n">
         <v>17.302023732283</v>
       </c>
-      <c r="I11" t="n">
+      <c r="P11" t="n">
         <v>19.0766961928649</v>
       </c>
-      <c r="J11" t="n">
+      <c r="Q11" t="n">
         <v>40131.1862089296</v>
       </c>
-      <c r="K11" t="n">
+      <c r="R11" t="n">
         <v>38680.0402145173</v>
       </c>
-      <c r="L11" t="n">
+      <c r="S11" t="n">
         <v>103.751666198805</v>
       </c>
-      <c r="M11" t="n">
+      <c r="T11" t="n">
         <v>-3.61161388417453</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>105</v>
-      </c>
-      <c r="B12" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="C12" t="n">
+        <v>223</v>
+      </c>
+      <c r="B12" t="s">
+        <v>211</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s">
+        <v>221</v>
+      </c>
+      <c r="E12" t="s">
+        <v>222</v>
+      </c>
+      <c r="F12" t="s">
+        <v>217</v>
+      </c>
+      <c r="G12" t="s">
+        <v>84</v>
+      </c>
+      <c r="H12" t="s">
+        <v>215</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="J12" t="n">
         <v>-0.39343495744554</v>
       </c>
-      <c r="D12" t="n">
+      <c r="K12" t="n">
         <v>0.679965559137567</v>
       </c>
-      <c r="E12" t="n">
+      <c r="L12" t="n">
         <v>2.73951091646933</v>
       </c>
-      <c r="F12" t="n">
+      <c r="M12" t="n">
         <v>0.025999999993833</v>
       </c>
-      <c r="G12" t="n">
+      <c r="N12" t="n">
         <v>0.0250830258410366</v>
       </c>
-      <c r="H12" t="n">
+      <c r="O12" t="n">
         <v>17.2495953099153</v>
       </c>
-      <c r="I12" t="n">
+      <c r="P12" t="n">
         <v>19.0774206742659</v>
       </c>
-      <c r="J12" t="n">
+      <c r="Q12" t="n">
         <v>40197.0702416694</v>
       </c>
-      <c r="K12" t="n">
+      <c r="R12" t="n">
         <v>38683.5986842421</v>
       </c>
-      <c r="L12" t="n">
+      <c r="S12" t="n">
         <v>103.912437334957</v>
       </c>
-      <c r="M12" t="n">
+      <c r="T12" t="n">
         <v>-3.45084274802267</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B13" t="n">
-        <v>0.026</v>
-      </c>
-      <c r="C13" t="n">
+        <v>224</v>
+      </c>
+      <c r="B13" t="s">
+        <v>211</v>
+      </c>
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" t="s">
+        <v>221</v>
+      </c>
+      <c r="E13" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" t="s">
+        <v>219</v>
+      </c>
+      <c r="G13" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" t="s">
+        <v>215</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="J13" t="n">
         <v>-0.284616104485266</v>
       </c>
-      <c r="D13" t="n">
+      <c r="K13" t="n">
         <v>0.681607207302063</v>
       </c>
-      <c r="E13" t="n">
+      <c r="L13" t="n">
         <v>2.74116043260915</v>
       </c>
-      <c r="F13" t="n">
+      <c r="M13" t="n">
         <v>0.0260000000040048</v>
       </c>
-      <c r="G13" t="n">
+      <c r="N13" t="n">
         <v>0.0251312519632405</v>
       </c>
-      <c r="H13" t="n">
+      <c r="O13" t="n">
         <v>17.3584141628755</v>
       </c>
-      <c r="I13" t="n">
+      <c r="P13" t="n">
         <v>19.0759169245472</v>
       </c>
-      <c r="J13" t="n">
+      <c r="Q13" t="n">
         <v>40060.3358463092</v>
       </c>
-      <c r="K13" t="n">
+      <c r="R13" t="n">
         <v>38676.2131084794</v>
       </c>
-      <c r="L13" t="n">
+      <c r="S13" t="n">
         <v>103.578744211455</v>
       </c>
-      <c r="M13" t="n">
+      <c r="T13" t="n">
         <v>-3.7845358715247</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>147</v>
-      </c>
-      <c r="B14" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="C14" t="n">
+        <v>225</v>
+      </c>
+      <c r="B14" t="s">
+        <v>221</v>
+      </c>
+      <c r="C14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" t="s">
+        <v>212</v>
+      </c>
+      <c r="E14" t="s">
+        <v>213</v>
+      </c>
+      <c r="F14" t="s">
+        <v>214</v>
+      </c>
+      <c r="G14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" t="s">
+        <v>215</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="J14" t="n">
         <v>-0.283540256177145</v>
       </c>
-      <c r="D14" t="n">
+      <c r="K14" t="n">
         <v>1.39662743424176</v>
       </c>
-      <c r="E14" t="n">
+      <c r="L14" t="n">
         <v>3.45960755796053</v>
       </c>
-      <c r="F14" t="n">
+      <c r="M14" t="n">
         <v>0.0330000000117017</v>
       </c>
-      <c r="G14" t="n">
+      <c r="N14" t="n">
         <v>0.0325754763608046</v>
       </c>
-      <c r="H14" t="n">
+      <c r="O14" t="n">
         <v>17.3594900111837</v>
       </c>
-      <c r="I14" t="n">
+      <c r="P14" t="n">
         <v>18.4209583966705</v>
       </c>
-      <c r="J14" t="n">
+      <c r="Q14" t="n">
         <v>39513.8980566219</v>
       </c>
-      <c r="K14" t="n">
+      <c r="R14" t="n">
         <v>39972.2645009952</v>
       </c>
-      <c r="L14" t="n">
+      <c r="S14" t="n">
         <v>98.853288773865</v>
       </c>
-      <c r="M14" t="n">
+      <c r="T14" t="n">
         <v>-8.50999130911495</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>148</v>
-      </c>
-      <c r="B15" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="C15" t="n">
+        <v>226</v>
+      </c>
+      <c r="B15" t="s">
+        <v>221</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" t="s">
+        <v>212</v>
+      </c>
+      <c r="E15" t="s">
+        <v>213</v>
+      </c>
+      <c r="F15" t="s">
+        <v>217</v>
+      </c>
+      <c r="G15" t="s">
+        <v>84</v>
+      </c>
+      <c r="H15" t="s">
+        <v>215</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="J15" t="n">
         <v>-0.385280365831578</v>
       </c>
-      <c r="D15" t="n">
+      <c r="K15" t="n">
         <v>1.39508028750381</v>
       </c>
-      <c r="E15" t="n">
+      <c r="L15" t="n">
         <v>3.45805299616704</v>
       </c>
-      <c r="F15" t="n">
+      <c r="M15" t="n">
         <v>0.0329999999996382</v>
       </c>
-      <c r="G15" t="n">
+      <c r="N15" t="n">
         <v>0.0325299861026989</v>
       </c>
-      <c r="H15" t="n">
+      <c r="O15" t="n">
         <v>17.2577499015292</v>
       </c>
-      <c r="I15" t="n">
+      <c r="P15" t="n">
         <v>18.4223755830824</v>
       </c>
-      <c r="J15" t="n">
+      <c r="Q15" t="n">
         <v>39644.7519768505</v>
       </c>
-      <c r="K15" t="n">
+      <c r="R15" t="n">
         <v>39979.4035623777</v>
       </c>
-      <c r="L15" t="n">
+      <c r="S15" t="n">
         <v>99.1629400248429</v>
       </c>
-      <c r="M15" t="n">
+      <c r="T15" t="n">
         <v>-8.20034005813699</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>149</v>
-      </c>
-      <c r="B16" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="C16" t="n">
+        <v>227</v>
+      </c>
+      <c r="B16" t="s">
+        <v>221</v>
+      </c>
+      <c r="C16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" t="s">
+        <v>212</v>
+      </c>
+      <c r="E16" t="s">
+        <v>213</v>
+      </c>
+      <c r="F16" t="s">
+        <v>219</v>
+      </c>
+      <c r="G16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" t="s">
+        <v>215</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="J16" t="n">
         <v>-0.166857854616306</v>
       </c>
-      <c r="D16" t="n">
+      <c r="K16" t="n">
         <v>1.39840198010221</v>
       </c>
-      <c r="E16" t="n">
+      <c r="L16" t="n">
         <v>3.46139060873896</v>
       </c>
-      <c r="F16" t="n">
+      <c r="M16" t="n">
         <v>0.0330000000049406</v>
       </c>
-      <c r="G16" t="n">
+      <c r="N16" t="n">
         <v>0.0326276584589438</v>
       </c>
-      <c r="H16" t="n">
+      <c r="O16" t="n">
         <v>17.4761724127445</v>
       </c>
-      <c r="I16" t="n">
+      <c r="P16" t="n">
         <v>18.4193329126623</v>
       </c>
-      <c r="J16" t="n">
+      <c r="Q16" t="n">
         <v>39363.8791656078</v>
       </c>
-      <c r="K16" t="n">
+      <c r="R16" t="n">
         <v>39964.0781350212</v>
       </c>
-      <c r="L16" t="n">
+      <c r="S16" t="n">
         <v>98.4981538485999</v>
       </c>
-      <c r="M16" t="n">
+      <c r="T16" t="n">
         <v>-8.86512623438001</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>107</v>
-      </c>
-      <c r="B17" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="C17" t="n">
+        <v>228</v>
+      </c>
+      <c r="B17" t="s">
+        <v>221</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" t="s">
+        <v>221</v>
+      </c>
+      <c r="E17" t="s">
+        <v>222</v>
+      </c>
+      <c r="F17" t="s">
+        <v>214</v>
+      </c>
+      <c r="G17" t="s">
+        <v>88</v>
+      </c>
+      <c r="H17" t="s">
+        <v>215</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="J17" t="n">
         <v>-0.757552904199768</v>
       </c>
-      <c r="D17" t="n">
+      <c r="K17" t="n">
         <v>1.38942041792633</v>
       </c>
-      <c r="E17" t="n">
+      <c r="L17" t="n">
         <v>3.45236600036662</v>
       </c>
-      <c r="F17" t="n">
+      <c r="M17" t="n">
         <v>0.033000000005794</v>
       </c>
-      <c r="G17" t="n">
+      <c r="N17" t="n">
         <v>0.0323636079372183</v>
       </c>
-      <c r="H17" t="n">
+      <c r="O17" t="n">
         <v>16.885477363161</v>
       </c>
-      <c r="I17" t="n">
+      <c r="P17" t="n">
         <v>18.4275600236154</v>
       </c>
-      <c r="J17" t="n">
+      <c r="Q17" t="n">
         <v>40123.9219589833</v>
       </c>
-      <c r="K17" t="n">
+      <c r="R17" t="n">
         <v>40005.5340988797</v>
       </c>
-      <c r="L17" t="n">
+      <c r="S17" t="n">
         <v>100.295928707791</v>
       </c>
-      <c r="M17" t="n">
+      <c r="T17" t="n">
         <v>-7.06735137518913</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="C18" t="n">
+        <v>229</v>
+      </c>
+      <c r="B18" t="s">
+        <v>221</v>
+      </c>
+      <c r="C18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" t="s">
+        <v>221</v>
+      </c>
+      <c r="E18" t="s">
+        <v>222</v>
+      </c>
+      <c r="F18" t="s">
+        <v>217</v>
+      </c>
+      <c r="G18" t="s">
+        <v>84</v>
+      </c>
+      <c r="H18" t="s">
+        <v>215</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="J18" t="n">
         <v>-0.854986673689603</v>
       </c>
-      <c r="D18" t="n">
+      <c r="K18" t="n">
         <v>1.3879393895631</v>
       </c>
-      <c r="E18" t="n">
+      <c r="L18" t="n">
         <v>3.45087787383533</v>
       </c>
-      <c r="F18" t="n">
+      <c r="M18" t="n">
         <v>0.03300000000106</v>
       </c>
-      <c r="G18" t="n">
+      <c r="N18" t="n">
         <v>0.032320081334005</v>
       </c>
-      <c r="H18" t="n">
+      <c r="O18" t="n">
         <v>16.7880435936712</v>
       </c>
-      <c r="I18" t="n">
+      <c r="P18" t="n">
         <v>18.4289166455961</v>
       </c>
-      <c r="J18" t="n">
+      <c r="Q18" t="n">
         <v>40249.4292790266</v>
       </c>
-      <c r="K18" t="n">
+      <c r="R18" t="n">
         <v>40012.3753197882</v>
       </c>
-      <c r="L18" t="n">
+      <c r="S18" t="n">
         <v>100.592451603645</v>
       </c>
-      <c r="M18" t="n">
+      <c r="T18" t="n">
         <v>-6.77082847933534</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>109</v>
-      </c>
-      <c r="B19" t="n">
-        <v>0.033</v>
-      </c>
-      <c r="C19" t="n">
+        <v>230</v>
+      </c>
+      <c r="B19" t="s">
+        <v>221</v>
+      </c>
+      <c r="C19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" t="s">
+        <v>221</v>
+      </c>
+      <c r="E19" t="s">
+        <v>222</v>
+      </c>
+      <c r="F19" t="s">
+        <v>219</v>
+      </c>
+      <c r="G19" t="s">
+        <v>90</v>
+      </c>
+      <c r="H19" t="s">
+        <v>215</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="J19" t="n">
         <v>-0.644506630947547</v>
       </c>
-      <c r="D19" t="n">
+      <c r="K19" t="n">
         <v>1.39113892291695</v>
       </c>
-      <c r="E19" t="n">
+      <c r="L19" t="n">
         <v>3.45409274168651</v>
       </c>
-      <c r="F19" t="n">
+      <c r="M19" t="n">
         <v>0.0330000000329154</v>
       </c>
-      <c r="G19" t="n">
+      <c r="N19" t="n">
         <v>0.0324141190847596</v>
       </c>
-      <c r="H19" t="n">
+      <c r="O19" t="n">
         <v>16.9985236364132</v>
       </c>
-      <c r="I19" t="n">
+      <c r="P19" t="n">
         <v>18.425985873044</v>
       </c>
-      <c r="J19" t="n">
+      <c r="Q19" t="n">
         <v>39978.3534254477</v>
       </c>
-      <c r="K19" t="n">
+      <c r="R19" t="n">
         <v>39997.5977837826</v>
       </c>
-      <c r="L19" t="n">
+      <c r="S19" t="n">
         <v>99.9518862146699</v>
       </c>
-      <c r="M19" t="n">
+      <c r="T19" t="n">
         <v>-7.41139386831006</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>141</v>
-      </c>
-      <c r="B20" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C20" t="n">
+        <v>231</v>
+      </c>
+      <c r="B20" t="s">
+        <v>232</v>
+      </c>
+      <c r="C20" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" t="s">
+        <v>212</v>
+      </c>
+      <c r="E20" t="s">
+        <v>213</v>
+      </c>
+      <c r="F20" t="s">
+        <v>214</v>
+      </c>
+      <c r="G20" t="s">
+        <v>88</v>
+      </c>
+      <c r="H20" t="s">
+        <v>215</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J20" t="n">
         <v>-0.0254857052549629</v>
       </c>
-      <c r="D20" t="n">
+      <c r="K20" t="n">
         <v>0.07282989908791</v>
       </c>
-      <c r="E20" t="n">
+      <c r="L20" t="n">
         <v>2.12946541953578</v>
       </c>
-      <c r="F20" t="n">
+      <c r="M20" t="n">
         <v>0.0199999999856091</v>
       </c>
-      <c r="G20" t="n">
+      <c r="N20" t="n">
         <v>0.0188705028858045</v>
       </c>
-      <c r="H20" t="n">
+      <c r="O20" t="n">
         <v>17.6175445621058</v>
       </c>
-      <c r="I20" t="n">
+      <c r="P20" t="n">
         <v>19.6335569388714</v>
       </c>
-      <c r="J20" t="n">
+      <c r="Q20" t="n">
         <v>40181.7693932306</v>
       </c>
-      <c r="K20" t="n">
+      <c r="R20" t="n">
         <v>37574.6852115126</v>
       </c>
-      <c r="L20" t="n">
+      <c r="S20" t="n">
         <v>106.938405916224</v>
       </c>
-      <c r="M20" t="n">
+      <c r="T20" t="n">
         <v>-0.424874166756325</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>142</v>
-      </c>
-      <c r="B21" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C21" t="n">
+        <v>233</v>
+      </c>
+      <c r="B21" t="s">
+        <v>232</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" t="s">
+        <v>212</v>
+      </c>
+      <c r="E21" t="s">
+        <v>213</v>
+      </c>
+      <c r="F21" t="s">
+        <v>217</v>
+      </c>
+      <c r="G21" t="s">
+        <v>84</v>
+      </c>
+      <c r="H21" t="s">
+        <v>215</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J21" t="n">
         <v>-0.0346378988383578</v>
       </c>
-      <c r="D21" t="n">
+      <c r="K21" t="n">
         <v>0.0726927356922062</v>
       </c>
-      <c r="E21" t="n">
+      <c r="L21" t="n">
         <v>2.12932759875306</v>
       </c>
-      <c r="F21" t="n">
+      <c r="M21" t="n">
         <v>0.0200000000002583</v>
       </c>
-      <c r="G21" t="n">
+      <c r="N21" t="n">
         <v>0.0188664753834344</v>
       </c>
-      <c r="H21" t="n">
+      <c r="O21" t="n">
         <v>17.6083923685224</v>
       </c>
-      <c r="I21" t="n">
+      <c r="P21" t="n">
         <v>19.6336825805419</v>
       </c>
-      <c r="J21" t="n">
+      <c r="Q21" t="n">
         <v>40193.0299894161</v>
       </c>
-      <c r="K21" t="n">
+      <c r="R21" t="n">
         <v>37575.2885179576</v>
       </c>
-      <c r="L21" t="n">
+      <c r="S21" t="n">
         <v>106.966657009719</v>
       </c>
-      <c r="M21" t="n">
+      <c r="T21" t="n">
         <v>-0.396623073260784</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>143</v>
-      </c>
-      <c r="B22" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C22" t="n">
+        <v>234</v>
+      </c>
+      <c r="B22" t="s">
+        <v>232</v>
+      </c>
+      <c r="C22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" t="s">
+        <v>212</v>
+      </c>
+      <c r="E22" t="s">
+        <v>213</v>
+      </c>
+      <c r="F22" t="s">
+        <v>219</v>
+      </c>
+      <c r="G22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H22" t="s">
+        <v>215</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J22" t="n">
         <v>-0.0162341236259994</v>
       </c>
-      <c r="D22" t="n">
+      <c r="K22" t="n">
         <v>0.0729685533773562</v>
       </c>
-      <c r="E22" t="n">
+      <c r="L22" t="n">
         <v>2.1296047383577</v>
       </c>
-      <c r="F22" t="n">
+      <c r="M22" t="n">
         <v>0.0199999999946143</v>
       </c>
-      <c r="G22" t="n">
+      <c r="N22" t="n">
         <v>0.0188745743566012</v>
       </c>
-      <c r="H22" t="n">
+      <c r="O22" t="n">
         <v>17.6267961437348</v>
       </c>
-      <c r="I22" t="n">
+      <c r="P22" t="n">
         <v>19.6334299315423</v>
       </c>
-      <c r="J22" t="n">
+      <c r="Q22" t="n">
         <v>40170.3868449224</v>
       </c>
-      <c r="K22" t="n">
+      <c r="R22" t="n">
         <v>37574.0753540371</v>
       </c>
-      <c r="L22" t="n">
+      <c r="S22" t="n">
         <v>106.909847990727</v>
       </c>
-      <c r="M22" t="n">
+      <c r="T22" t="n">
         <v>-0.453432092252598</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B23" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C23" t="n">
+        <v>235</v>
+      </c>
+      <c r="B23" t="s">
+        <v>232</v>
+      </c>
+      <c r="C23" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" t="s">
+        <v>221</v>
+      </c>
+      <c r="E23" t="s">
+        <v>222</v>
+      </c>
+      <c r="F23" t="s">
+        <v>214</v>
+      </c>
+      <c r="G23" t="s">
+        <v>88</v>
+      </c>
+      <c r="H23" t="s">
+        <v>215</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J23" t="n">
         <v>-0.0822707695848912</v>
       </c>
-      <c r="D23" t="n">
+      <c r="K23" t="n">
         <v>0.0719788820351838</v>
       </c>
-      <c r="E23" t="n">
+      <c r="L23" t="n">
         <v>2.12861032378866</v>
       </c>
-      <c r="F23" t="n">
+      <c r="M23" t="n">
         <v>0.0199999999895371</v>
       </c>
-      <c r="G23" t="n">
+      <c r="N23" t="n">
         <v>0.0188455148203448</v>
       </c>
-      <c r="H23" t="n">
+      <c r="O23" t="n">
         <v>17.5607594977759</v>
       </c>
-      <c r="I23" t="n">
+      <c r="P23" t="n">
         <v>19.6343364704917</v>
       </c>
-      <c r="J23" t="n">
+      <c r="Q23" t="n">
         <v>40251.6415476907</v>
       </c>
-      <c r="K23" t="n">
+      <c r="R23" t="n">
         <v>37578.4285916403</v>
       </c>
-      <c r="L23" t="n">
+      <c r="S23" t="n">
         <v>107.113690104235</v>
       </c>
-      <c r="M23" t="n">
+      <c r="T23" t="n">
         <v>-0.249589978745206</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>102</v>
-      </c>
-      <c r="B24" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C24" t="n">
+        <v>236</v>
+      </c>
+      <c r="B24" t="s">
+        <v>232</v>
+      </c>
+      <c r="C24" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" t="s">
+        <v>221</v>
+      </c>
+      <c r="E24" t="s">
+        <v>222</v>
+      </c>
+      <c r="F24" t="s">
+        <v>217</v>
+      </c>
+      <c r="G24" t="s">
+        <v>84</v>
+      </c>
+      <c r="H24" t="s">
+        <v>215</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J24" t="n">
         <v>-0.0913934496556274</v>
       </c>
-      <c r="D24" t="n">
+      <c r="K24" t="n">
         <v>0.0718421678274633</v>
       </c>
-      <c r="E24" t="n">
+      <c r="L24" t="n">
         <v>2.12847295434675</v>
       </c>
-      <c r="F24" t="n">
+      <c r="M24" t="n">
         <v>0.0199999999835945</v>
       </c>
-      <c r="G24" t="n">
+      <c r="N24" t="n">
         <v>0.0188415006548048</v>
       </c>
-      <c r="H24" t="n">
+      <c r="O24" t="n">
         <v>17.5516368177052</v>
       </c>
-      <c r="I24" t="n">
+      <c r="P24" t="n">
         <v>19.634461700706</v>
       </c>
-      <c r="J24" t="n">
+      <c r="Q24" t="n">
         <v>40262.867909424</v>
       </c>
-      <c r="K24" t="n">
+      <c r="R24" t="n">
         <v>37579.0300044955</v>
       </c>
-      <c r="L24" t="n">
+      <c r="S24" t="n">
         <v>107.141849868417</v>
       </c>
-      <c r="M24" t="n">
+      <c r="T24" t="n">
         <v>-0.221430214562915</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>103</v>
-      </c>
-      <c r="B25" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C25" t="n">
+        <v>237</v>
+      </c>
+      <c r="B25" t="s">
+        <v>232</v>
+      </c>
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" t="s">
+        <v>221</v>
+      </c>
+      <c r="E25" t="s">
+        <v>222</v>
+      </c>
+      <c r="F25" t="s">
+        <v>219</v>
+      </c>
+      <c r="G25" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" t="s">
+        <v>215</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="J25" t="n">
         <v>-0.0730537432937967</v>
       </c>
-      <c r="D25" t="n">
+      <c r="K25" t="n">
         <v>0.0721170116787752</v>
       </c>
-      <c r="E25" t="n">
+      <c r="L25" t="n">
         <v>2.12874911545025</v>
       </c>
-      <c r="F25" t="n">
+      <c r="M25" t="n">
         <v>0.0200000000202882</v>
       </c>
-      <c r="G25" t="n">
+      <c r="N25" t="n">
         <v>0.0188495706886871</v>
       </c>
-      <c r="H25" t="n">
+      <c r="O25" t="n">
         <v>17.569976524067</v>
       </c>
-      <c r="I25" t="n">
+      <c r="P25" t="n">
         <v>19.6342099437382</v>
       </c>
-      <c r="J25" t="n">
+      <c r="Q25" t="n">
         <v>40240.2994200197</v>
       </c>
-      <c r="K25" t="n">
+      <c r="R25" t="n">
         <v>37577.8209683877</v>
       </c>
-      <c r="L25" t="n">
+      <c r="S25" t="n">
         <v>107.085239066607</v>
       </c>
-      <c r="M25" t="n">
+      <c r="T25" t="n">
         <v>-0.278041016372569</v>
       </c>
     </row>
@@ -6551,13 +7069,13 @@
         <v>130</v>
       </c>
       <c r="C8" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D8" t="n">
-        <v>101.336467661375</v>
+        <v>-101.336467661375</v>
       </c>
       <c r="E8" t="n">
-        <v>0.368722591245188</v>
+        <v>-0.368722591245188</v>
       </c>
       <c r="F8" t="n">
         <v>8.36632274246801</v>
@@ -6639,13 +7157,13 @@
         <v>130</v>
       </c>
       <c r="C12" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D12" t="n">
-        <v>100.250164843803</v>
+        <v>-100.250164843803</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.717580226326447</v>
+        <v>0.717580226326447</v>
       </c>
       <c r="F12" t="n">
         <v>8.36632274246801</v>
@@ -6727,13 +7245,13 @@
         <v>130</v>
       </c>
       <c r="C16" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D16" t="n">
-        <v>102.420857738251</v>
+        <v>-102.420857738251</v>
       </c>
       <c r="E16" t="n">
-        <v>1.45311266812115</v>
+        <v>-1.45311266812115</v>
       </c>
       <c r="F16" t="n">
         <v>8.36632274246801</v>
@@ -6815,13 +7333,13 @@
         <v>130</v>
       </c>
       <c r="C20" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D20" t="n">
-        <v>100.344407038839</v>
+        <v>-100.344407038839</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.623338031290842</v>
+        <v>0.623338031290842</v>
       </c>
       <c r="F20" t="n">
         <v>36.658756959679</v>
@@ -6903,13 +7421,13 @@
         <v>130</v>
       </c>
       <c r="C24" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D24" t="n">
-        <v>93.6888221250927</v>
+        <v>-93.6888221250927</v>
       </c>
       <c r="E24" t="n">
-        <v>-7.27892294503704</v>
+        <v>7.27892294503704</v>
       </c>
       <c r="F24" t="n">
         <v>36.658756959679</v>
@@ -6991,13 +7509,13 @@
         <v>130</v>
       </c>
       <c r="C28" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D28" t="n">
-        <v>106.858683756629</v>
+        <v>-106.858683756629</v>
       </c>
       <c r="E28" t="n">
-        <v>5.89093868649896</v>
+        <v>-5.89093868649896</v>
       </c>
       <c r="F28" t="n">
         <v>36.658756959679</v>
@@ -7079,13 +7597,13 @@
         <v>130</v>
       </c>
       <c r="C32" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D32" t="n">
-        <v>101.895654142962</v>
+        <v>-101.895654142962</v>
       </c>
       <c r="E32" t="n">
-        <v>0.927909072832591</v>
+        <v>-0.927909072832591</v>
       </c>
       <c r="F32" t="n">
         <v>84.0011710987443</v>
@@ -7167,13 +7685,13 @@
         <v>130</v>
       </c>
       <c r="C36" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D36" t="n">
-        <v>88.5670719690749</v>
+        <v>-88.5670719690749</v>
       </c>
       <c r="E36" t="n">
-        <v>-12.4006731010548</v>
+        <v>12.4006731010548</v>
       </c>
       <c r="F36" t="n">
         <v>84.0011710987443</v>
@@ -7255,13 +7773,13 @@
         <v>130</v>
       </c>
       <c r="C40" t="n">
-        <v>100.96774507013</v>
+        <v>-100.96774507013</v>
       </c>
       <c r="D40" t="n">
-        <v>114.468920469056</v>
+        <v>-114.468920469056</v>
       </c>
       <c r="E40" t="n">
-        <v>13.5011753989266</v>
+        <v>-13.5011753989266</v>
       </c>
       <c r="F40" t="n">
         <v>84.0011710987443</v>
@@ -7482,7 +8000,7 @@
         <v>8.16574765183793</v>
       </c>
       <c r="E13" t="n">
-        <v>28.4967461669466</v>
+        <v>28.4967461669469</v>
       </c>
     </row>
     <row r="14">
@@ -7499,7 +8017,7 @@
         <v>4.73452914373081</v>
       </c>
       <c r="E14" t="n">
-        <v>28.4967461669466</v>
+        <v>28.4967461669469</v>
       </c>
     </row>
     <row r="15">
@@ -7516,7 +8034,7 @@
         <v>11.6324516198077</v>
       </c>
       <c r="E15" t="n">
-        <v>28.4967461669466</v>
+        <v>28.4967461669469</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
results: v1.0.1 bundles and the with/without-erratum result set
Regenerate the 2030 bundles, figure suite and paper exhibit workbook
from the v1.0.1 run (both fixes). Add results/erratum_v1.0.1/: full CSV
results for four runs (A v1.0.0 as published, B Karger fix only, C CBO
fix only, D v1.0.1) plus comparison tables attributing every number to
each fix, and code/erratum_v1_0_1_export.R that builds them. Run A
reproduces the published v1.0.0 exactly (inputs byte-identical, every
bundle sheet within 1e-9).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/figures/2030/paper_figure_data_2030.xlsx
+++ b/results/figures/2030/paper_figure_data_2030.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">AI-Fiscal — paper exhibits (FY 2030)</t>
   </si>
   <si>
-    <t xml:space="preserve">July 2026</t>
+    <t xml:space="preserve">October 2026</t>
   </si>
   <si>
     <t xml:space="preserve">The Budget Lab at Yale</t>
@@ -212,10 +212,10 @@
     <t xml:space="preserve">0.45</t>
   </si>
   <si>
-    <t xml:space="preserve">0.462</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.487</t>
+    <t xml:space="preserve">0.46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.48</t>
   </si>
   <si>
     <t xml:space="preserve">2030 labor share (theta_1_L)</t>
@@ -224,16 +224,16 @@
     <t xml:space="preserve">0.55</t>
   </si>
   <si>
-    <t xml:space="preserve">0.538</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.513</t>
+    <t xml:space="preserve">0.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.52</t>
   </si>
   <si>
     <t xml:space="preserve">Derived growth bumps</t>
   </si>
   <si>
-    <t xml:space="preserve">Cumulative over the Karger 5-year horizon, above the CBO no-AI baseline path.</t>
+    <t xml:space="preserve">Cumulative over the Karger 5-year horizon, above the CBO baseline path (which already embeds a small AI effect: +0.1 pp/yr TFP).</t>
   </si>
   <si>
     <t xml:space="preserve">GDP                  (g_y)</t>
@@ -254,10 +254,10 @@
     <t xml:space="preserve">0.0172117163991912</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0754166612691227</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.172812402611785</t>
+    <t xml:space="preserve">0.0707611778870052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.155954729473628</t>
   </si>
   <si>
     <t xml:space="preserve">Labor                (L_1/L_0 - 1)</t>
@@ -266,10 +266,10 @@
     <t xml:space="preserve">-0.00315288252772006</t>
   </si>
   <si>
-    <t xml:space="preserve">0.00411646532678422</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.00943271239531995</t>
+    <t xml:space="preserve">0.00784924029082745</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00408380030104216</t>
   </si>
   <si>
     <t xml:space="preserve">Labor-income inequality parameter (lambda)</t>
@@ -2571,7 +2571,7 @@
         <v>2021</v>
       </c>
       <c r="B76" t="n">
-        <v>0.0235382702054906</v>
+        <v>0.0237573082522044</v>
       </c>
       <c r="C76"/>
       <c r="D76" t="n">
@@ -2589,7 +2589,7 @@
         <v>2022</v>
       </c>
       <c r="B77" t="n">
-        <v>0.0236682162326723</v>
+        <v>0.0237025923488549</v>
       </c>
       <c r="C77"/>
       <c r="D77" t="n">
@@ -2607,7 +2607,7 @@
         <v>2023</v>
       </c>
       <c r="B78" t="n">
-        <v>0.0236057828903334</v>
+        <v>0.0236094464296709</v>
       </c>
       <c r="C78"/>
       <c r="D78" t="n">
@@ -2625,7 +2625,7 @@
         <v>2024</v>
       </c>
       <c r="B79" t="n">
-        <v>0.0240135318044857</v>
+        <v>0.0243254433617899</v>
       </c>
       <c r="C79"/>
       <c r="D79" t="n">
@@ -2643,10 +2643,10 @@
         <v>2025</v>
       </c>
       <c r="B80" t="n">
-        <v>0.0323891425079967</v>
+        <v>0.0331663413820539</v>
       </c>
       <c r="C80" t="n">
-        <v>0.0323891425079967</v>
+        <v>0.0331663413820539</v>
       </c>
       <c r="D80" t="n">
         <v>0.02</v>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="B81"/>
       <c r="C81" t="n">
-        <v>0.024801029860323</v>
+        <v>0.0253591906876665</v>
       </c>
       <c r="D81" t="n">
         <v>0.02</v>
@@ -2682,7 +2682,7 @@
       </c>
       <c r="B82"/>
       <c r="C82" t="n">
-        <v>0.0233832477437041</v>
+        <v>0.0241260705015787</v>
       </c>
       <c r="D82" t="n">
         <v>0.02</v>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="B83"/>
       <c r="C83" t="n">
-        <v>0.0211669660683029</v>
+        <v>0.0219405014030229</v>
       </c>
       <c r="D83" t="n">
         <v>0.02</v>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="B84"/>
       <c r="C84" t="n">
-        <v>0.0192251712311784</v>
+        <v>0.0196904585479317</v>
       </c>
       <c r="D84" t="n">
         <v>0.02</v>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="B85"/>
       <c r="C85" t="n">
-        <v>0.0186242328589671</v>
+        <v>0.0186242328589675</v>
       </c>
       <c r="D85" t="n">
         <v>0.02</v>
@@ -2790,7 +2790,7 @@
       </c>
       <c r="B88"/>
       <c r="C88" t="n">
-        <v>0.0178399181283311</v>
+        <v>0.0178399181283307</v>
       </c>
       <c r="D88" t="n">
         <v>0.02</v>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="B89"/>
       <c r="C89" t="n">
-        <v>0.0178399181283311</v>
+        <v>0.0178399181283307</v>
       </c>
       <c r="D89" t="n">
         <v>0.02</v>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="B90"/>
       <c r="C90" t="n">
-        <v>0.0178399181283311</v>
+        <v>0.0178399181283307</v>
       </c>
       <c r="D90" t="n">
         <v>0.02</v>
@@ -2922,10 +2922,10 @@
         <v>0.55</v>
       </c>
       <c r="D7" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E7" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="8">
@@ -2939,10 +2939,10 @@
         <v>0.55</v>
       </c>
       <c r="D8" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E8" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="9">
@@ -2956,10 +2956,10 @@
         <v>0.55</v>
       </c>
       <c r="D9" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E9" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="10">
@@ -2973,10 +2973,10 @@
         <v>0.55</v>
       </c>
       <c r="D10" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E10" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="11">
@@ -2990,10 +2990,10 @@
         <v>0.55</v>
       </c>
       <c r="D11" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E11" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="12">
@@ -3007,10 +3007,10 @@
         <v>0.55</v>
       </c>
       <c r="D12" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E12" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="13">
@@ -3024,10 +3024,10 @@
         <v>0.55</v>
       </c>
       <c r="D13" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E13" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="14">
@@ -3041,10 +3041,10 @@
         <v>0.55</v>
       </c>
       <c r="D14" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E14" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="15">
@@ -3058,10 +3058,10 @@
         <v>0.55</v>
       </c>
       <c r="D15" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E15" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="16">
@@ -3075,10 +3075,10 @@
         <v>0.55</v>
       </c>
       <c r="D16" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E16" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="17">
@@ -3092,10 +3092,10 @@
         <v>0.55</v>
       </c>
       <c r="D17" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E17" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="18">
@@ -3109,10 +3109,10 @@
         <v>0.55</v>
       </c>
       <c r="D18" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E18" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="19">
@@ -3126,10 +3126,10 @@
         <v>0.55</v>
       </c>
       <c r="D19" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E19" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="20">
@@ -3143,10 +3143,10 @@
         <v>0.55</v>
       </c>
       <c r="D20" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E20" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="21">
@@ -3160,10 +3160,10 @@
         <v>0.55</v>
       </c>
       <c r="D21" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E21" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="22">
@@ -3177,10 +3177,10 @@
         <v>0.55</v>
       </c>
       <c r="D22" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E22" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="23">
@@ -3194,10 +3194,10 @@
         <v>0.55</v>
       </c>
       <c r="D23" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E23" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="24">
@@ -3211,10 +3211,10 @@
         <v>0.55</v>
       </c>
       <c r="D24" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E24" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="25">
@@ -3228,10 +3228,10 @@
         <v>0.55</v>
       </c>
       <c r="D25" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E25" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="26">
@@ -3245,10 +3245,10 @@
         <v>0.55</v>
       </c>
       <c r="D26" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E26" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="27">
@@ -3262,10 +3262,10 @@
         <v>0.55</v>
       </c>
       <c r="D27" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E27" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="28">
@@ -3279,10 +3279,10 @@
         <v>0.55</v>
       </c>
       <c r="D28" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E28" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="29">
@@ -3296,10 +3296,10 @@
         <v>0.55</v>
       </c>
       <c r="D29" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E29" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="30">
@@ -3313,10 +3313,10 @@
         <v>0.55</v>
       </c>
       <c r="D30" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E30" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="31">
@@ -3330,10 +3330,10 @@
         <v>0.55</v>
       </c>
       <c r="D31" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E31" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="32">
@@ -3347,10 +3347,10 @@
         <v>0.55</v>
       </c>
       <c r="D32" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E32" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="33">
@@ -3364,10 +3364,10 @@
         <v>0.55</v>
       </c>
       <c r="D33" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E33" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="34">
@@ -3381,10 +3381,10 @@
         <v>0.55</v>
       </c>
       <c r="D34" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E34" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="35">
@@ -3398,10 +3398,10 @@
         <v>0.55</v>
       </c>
       <c r="D35" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E35" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="36">
@@ -3415,10 +3415,10 @@
         <v>0.55</v>
       </c>
       <c r="D36" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E36" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="37">
@@ -3432,10 +3432,10 @@
         <v>0.55</v>
       </c>
       <c r="D37" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E37" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="38">
@@ -3449,10 +3449,10 @@
         <v>0.55</v>
       </c>
       <c r="D38" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E38" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="39">
@@ -3466,10 +3466,10 @@
         <v>0.55</v>
       </c>
       <c r="D39" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E39" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="40">
@@ -3483,10 +3483,10 @@
         <v>0.55</v>
       </c>
       <c r="D40" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E40" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="41">
@@ -3500,10 +3500,10 @@
         <v>0.55</v>
       </c>
       <c r="D41" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E41" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="42">
@@ -3517,10 +3517,10 @@
         <v>0.55</v>
       </c>
       <c r="D42" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E42" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="43">
@@ -3534,10 +3534,10 @@
         <v>0.55</v>
       </c>
       <c r="D43" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E43" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="44">
@@ -3551,10 +3551,10 @@
         <v>0.55</v>
       </c>
       <c r="D44" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E44" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="45">
@@ -3568,10 +3568,10 @@
         <v>0.55</v>
       </c>
       <c r="D45" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E45" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="46">
@@ -3585,10 +3585,10 @@
         <v>0.55</v>
       </c>
       <c r="D46" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E46" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="47">
@@ -3602,10 +3602,10 @@
         <v>0.55</v>
       </c>
       <c r="D47" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E47" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="48">
@@ -3619,10 +3619,10 @@
         <v>0.55</v>
       </c>
       <c r="D48" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E48" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="49">
@@ -3636,10 +3636,10 @@
         <v>0.55</v>
       </c>
       <c r="D49" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E49" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="50">
@@ -3653,10 +3653,10 @@
         <v>0.55</v>
       </c>
       <c r="D50" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E50" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="51">
@@ -3670,10 +3670,10 @@
         <v>0.55</v>
       </c>
       <c r="D51" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E51" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="52">
@@ -3687,10 +3687,10 @@
         <v>0.55</v>
       </c>
       <c r="D52" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E52" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="53">
@@ -3704,10 +3704,10 @@
         <v>0.55</v>
       </c>
       <c r="D53" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E53" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="54">
@@ -3721,10 +3721,10 @@
         <v>0.55</v>
       </c>
       <c r="D54" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E54" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="55">
@@ -3738,10 +3738,10 @@
         <v>0.55</v>
       </c>
       <c r="D55" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E55" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="56">
@@ -3755,10 +3755,10 @@
         <v>0.55</v>
       </c>
       <c r="D56" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E56" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="57">
@@ -3772,10 +3772,10 @@
         <v>0.55</v>
       </c>
       <c r="D57" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E57" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="58">
@@ -3789,10 +3789,10 @@
         <v>0.55</v>
       </c>
       <c r="D58" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E58" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="59">
@@ -3806,10 +3806,10 @@
         <v>0.55</v>
       </c>
       <c r="D59" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E59" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="60">
@@ -3823,10 +3823,10 @@
         <v>0.55</v>
       </c>
       <c r="D60" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E60" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="61">
@@ -3840,10 +3840,10 @@
         <v>0.55</v>
       </c>
       <c r="D61" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E61" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="62">
@@ -3857,10 +3857,10 @@
         <v>0.55</v>
       </c>
       <c r="D62" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E62" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="63">
@@ -3874,10 +3874,10 @@
         <v>0.55</v>
       </c>
       <c r="D63" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E63" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="64">
@@ -3891,10 +3891,10 @@
         <v>0.55</v>
       </c>
       <c r="D64" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E64" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="65">
@@ -3908,10 +3908,10 @@
         <v>0.55</v>
       </c>
       <c r="D65" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E65" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="66">
@@ -3925,10 +3925,10 @@
         <v>0.55</v>
       </c>
       <c r="D66" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E66" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="67">
@@ -3942,10 +3942,10 @@
         <v>0.55</v>
       </c>
       <c r="D67" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E67" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="68">
@@ -3959,10 +3959,10 @@
         <v>0.55</v>
       </c>
       <c r="D68" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E68" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="69">
@@ -3976,10 +3976,10 @@
         <v>0.55</v>
       </c>
       <c r="D69" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E69" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="70">
@@ -3993,10 +3993,10 @@
         <v>0.55</v>
       </c>
       <c r="D70" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E70" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="71">
@@ -4010,10 +4010,10 @@
         <v>0.55</v>
       </c>
       <c r="D71" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E71" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="72">
@@ -4027,10 +4027,10 @@
         <v>0.55</v>
       </c>
       <c r="D72" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E72" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="73">
@@ -4044,10 +4044,10 @@
         <v>0.55</v>
       </c>
       <c r="D73" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E73" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="74">
@@ -4061,10 +4061,10 @@
         <v>0.55</v>
       </c>
       <c r="D74" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E74" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="75">
@@ -4078,10 +4078,10 @@
         <v>0.55</v>
       </c>
       <c r="D75" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E75" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="76">
@@ -4095,10 +4095,10 @@
         <v>0.55</v>
       </c>
       <c r="D76" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E76" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="77">
@@ -4112,10 +4112,10 @@
         <v>0.55</v>
       </c>
       <c r="D77" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E77" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="78">
@@ -4129,10 +4129,10 @@
         <v>0.55</v>
       </c>
       <c r="D78" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E78" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="79">
@@ -4146,10 +4146,10 @@
         <v>0.55</v>
       </c>
       <c r="D79" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E79" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="80">
@@ -4163,10 +4163,10 @@
         <v>0.55</v>
       </c>
       <c r="D80" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E80" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="81">
@@ -4180,10 +4180,10 @@
         <v>0.55</v>
       </c>
       <c r="D81" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E81" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="82">
@@ -4197,10 +4197,10 @@
         <v>0.55</v>
       </c>
       <c r="D82" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E82" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="83">
@@ -4214,10 +4214,10 @@
         <v>0.55</v>
       </c>
       <c r="D83" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E83" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="84">
@@ -4231,10 +4231,10 @@
         <v>0.55</v>
       </c>
       <c r="D84" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E84" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="85">
@@ -4248,10 +4248,10 @@
         <v>0.55</v>
       </c>
       <c r="D85" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E85" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="86">
@@ -4259,16 +4259,16 @@
         <v>2026</v>
       </c>
       <c r="B86" t="n">
-        <v>0.53667739967801</v>
+        <v>0.53190046798596</v>
       </c>
       <c r="C86" t="n">
         <v>0.55</v>
       </c>
       <c r="D86" t="n">
-        <v>0.538</v>
+        <v>0.54</v>
       </c>
       <c r="E86" t="n">
-        <v>0.513</v>
+        <v>0.52</v>
       </c>
     </row>
   </sheetData>
@@ -4366,10 +4366,10 @@
         <v>104</v>
       </c>
       <c r="B7" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.623338031290842</v>
+        <v>-1.07849179806213</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -4378,34 +4378,34 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>62.9615182243424</v>
+        <v>69.0530073180144</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>4.91016033234359</v>
+        <v>9.3556340249479</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>68.4950165879764</v>
+        <v>79.4871331410241</v>
       </c>
       <c r="K7" t="n">
-        <v>52.7340772104844</v>
+        <v>49.4313684315475</v>
       </c>
       <c r="L7" t="n">
-        <v>0.0257895279983131</v>
+        <v>0.0480621953411173</v>
       </c>
       <c r="M7" t="n">
-        <v>15.7351498494936</v>
+        <v>30.0077025141354</v>
       </c>
       <c r="N7" t="n">
-        <v>105.153773547655</v>
+        <v>113.264608019879</v>
       </c>
       <c r="O7" t="n">
-        <v>362.908528570293</v>
+        <v>403.085723180422</v>
       </c>
     </row>
     <row r="8">
@@ -4413,10 +4413,10 @@
         <v>105</v>
       </c>
       <c r="B8" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="C8" t="n">
-        <v>-7.27892294503704</v>
+        <v>-7.74837234431591</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -4425,34 +4425,34 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>11.121816981813</v>
+        <v>17.064085764795</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>29.7880763576211</v>
+        <v>34.3343914073391</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>48.1888162844707</v>
+        <v>59.146849516449</v>
       </c>
       <c r="K8" t="n">
-        <v>52.7340772104844</v>
+        <v>49.4313684315475</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.0185880125118274</v>
+        <v>0.0038104265659058</v>
       </c>
       <c r="M8" t="n">
-        <v>-4.5266729135019</v>
+        <v>9.71167065833561</v>
       </c>
       <c r="N8" t="n">
-        <v>84.8475732441497</v>
+        <v>92.9243243953035</v>
       </c>
       <c r="O8" t="n">
-        <v>356.367497335003</v>
+        <v>396.519941774583</v>
       </c>
     </row>
     <row r="9">
@@ -4460,10 +4460,10 @@
         <v>106</v>
       </c>
       <c r="B9" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="C9" t="n">
-        <v>5.89093868649896</v>
+        <v>5.45111444954932</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -4472,34 +4472,34 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>117.235044082048</v>
+        <v>123.483438790769</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>-21.0083519114044</v>
+        <v>-16.6618761854836</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>90.3357534841434</v>
+        <v>101.370448155736</v>
       </c>
       <c r="K9" t="n">
-        <v>52.7340772104844</v>
+        <v>49.4313684315475</v>
       </c>
       <c r="L9" t="n">
-        <v>0.091387280644085</v>
+        <v>0.113857235893192</v>
       </c>
       <c r="M9" t="n">
-        <v>37.5102889930149</v>
+        <v>51.8252224882954</v>
       </c>
       <c r="N9" t="n">
-        <v>126.994510443822</v>
+        <v>135.147923034591</v>
       </c>
       <c r="O9" t="n">
-        <v>368.753060256702</v>
+        <v>408.951288056593</v>
       </c>
     </row>
     <row r="10">
@@ -4507,10 +4507,10 @@
         <v>107</v>
       </c>
       <c r="B10" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="C10" t="n">
-        <v>0.927909072832591</v>
+        <v>-0.737832220917753</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -4519,34 +4519,34 @@
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>98.9616612919495</v>
+        <v>120.740916836021</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>-11.2886702738613</v>
+        <v>4.87123295222636</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>86.7450819452543</v>
+        <v>126.349982009165</v>
       </c>
       <c r="K10" t="n">
-        <v>122.932200326053</v>
+        <v>110.676210036276</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.155147368337566</v>
+        <v>0.063487409624031</v>
       </c>
       <c r="M10" t="n">
-        <v>-36.0319710124613</v>
+        <v>15.6102845632649</v>
       </c>
       <c r="N10" t="n">
-        <v>170.746253043999</v>
+        <v>200.79414919708</v>
       </c>
       <c r="O10" t="n">
-        <v>535.921491163816</v>
+        <v>681.365966532718</v>
       </c>
     </row>
     <row r="11">
@@ -4554,10 +4554,10 @@
         <v>108</v>
       </c>
       <c r="B11" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="C11" t="n">
-        <v>-12.4006731010548</v>
+        <v>-14.1468765597672</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -4566,34 +4566,34 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>-1.37895589235222</v>
+        <v>19.3167426642071</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>36.6809936673592</v>
+        <v>53.5658418148544</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>47.7027108760613</v>
+        <v>87.0294610388273</v>
       </c>
       <c r="K11" t="n">
-        <v>122.932200326053</v>
+        <v>110.676210036276</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.504212762140014</v>
+        <v>-0.261336248324369</v>
       </c>
       <c r="M11" t="n">
-        <v>-74.7252766878519</v>
+        <v>-23.385412749124</v>
       </c>
       <c r="N11" t="n">
-        <v>131.703881974806</v>
+        <v>161.473628226743</v>
       </c>
       <c r="O11" t="n">
-        <v>522.1905576709</v>
+        <v>667.452005752053</v>
       </c>
     </row>
     <row r="12">
@@ -4601,10 +4601,10 @@
         <v>109</v>
       </c>
       <c r="B12" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="C12" t="n">
-        <v>13.5011753989266</v>
+        <v>11.9970284572449</v>
       </c>
       <c r="D12" t="n">
         <v>0</v>
@@ -4613,34 +4613,34 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>208.968910957338</v>
+        <v>231.870770165091</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>-63.4242465884479</v>
+        <v>-47.985752299868</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>132.043488969963</v>
+        <v>171.887989407977</v>
       </c>
       <c r="K12" t="n">
-        <v>122.932200326053</v>
+        <v>110.676210036276</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0815239017138083</v>
+        <v>0.288739502173485</v>
       </c>
       <c r="M12" t="n">
-        <v>9.02976474219577</v>
+        <v>60.9230398695281</v>
       </c>
       <c r="N12" t="n">
-        <v>216.044660068707</v>
+        <v>246.332156595892</v>
       </c>
       <c r="O12" t="n">
-        <v>546.8013758505</v>
+        <v>692.402195271912</v>
       </c>
     </row>
     <row r="13">
@@ -4648,7 +4648,7 @@
         <v>101</v>
       </c>
       <c r="B13" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="C13" t="n">
         <v>0.368722591245188</v>
@@ -4684,7 +4684,7 @@
         <v>-12.0475000680008</v>
       </c>
       <c r="N13" t="n">
-        <v>8.16574765183793</v>
+        <v>8.01534691145987</v>
       </c>
       <c r="O13" t="n">
         <v>18.4844202005042</v>
@@ -4695,7 +4695,7 @@
         <v>102</v>
       </c>
       <c r="B14" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="C14" t="n">
         <v>-0.717580226326447</v>
@@ -4731,7 +4731,7 @@
         <v>-15.4798500404941</v>
       </c>
       <c r="N14" t="n">
-        <v>4.73452914373081</v>
+        <v>4.58412840335275</v>
       </c>
       <c r="O14" t="n">
         <v>17.460016963887</v>
@@ -4742,7 +4742,7 @@
         <v>103</v>
       </c>
       <c r="B15" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="C15" t="n">
         <v>1.45311266812115</v>
@@ -4778,7 +4778,7 @@
         <v>-8.58025745691975</v>
       </c>
       <c r="N15" t="n">
-        <v>11.6324516198077</v>
+        <v>11.4820508794297</v>
       </c>
       <c r="O15" t="n">
         <v>19.4883121339044</v>
@@ -4969,37 +4969,37 @@
         <v>0.026</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.148558309057403</v>
+        <v>-0.147224992003586</v>
       </c>
       <c r="K8" t="n">
-        <v>0.683660008499217</v>
+        <v>0.683680125187522</v>
       </c>
       <c r="L8" t="n">
-        <v>2.74322307232682</v>
+        <v>2.74324328542894</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0259999999925518</v>
+        <v>0.0259999999975653</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0251915636891986</v>
+        <v>0.0251921548070868</v>
       </c>
       <c r="O8" t="n">
-        <v>17.4944719583034</v>
+        <v>17.4958052753572</v>
       </c>
       <c r="P8" t="n">
-        <v>19.0740365586506</v>
+        <v>19.0740181317642</v>
       </c>
       <c r="Q8" t="n">
-        <v>39889.4428134478</v>
+        <v>39887.768495108</v>
       </c>
       <c r="R8" t="n">
-        <v>38666.9803218121</v>
+        <v>38666.8898495812</v>
       </c>
       <c r="S8" t="n">
-        <v>103.161515281156</v>
+        <v>103.157426548337</v>
       </c>
       <c r="T8" t="n">
-        <v>-4.20176480182364</v>
+        <v>-4.20585353464321</v>
       </c>
     </row>
     <row r="9">
@@ -5031,37 +5031,37 @@
         <v>0.026</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.201752970943184</v>
+        <v>-0.200419653889367</v>
       </c>
       <c r="K9" t="n">
-        <v>0.682857390632746</v>
+        <v>0.682877509815597</v>
       </c>
       <c r="L9" t="n">
-        <v>2.74241660773014</v>
+        <v>2.74243682333879</v>
       </c>
       <c r="M9" t="n">
-        <v>0.0259999999790508</v>
+        <v>0.0260000000087188</v>
       </c>
       <c r="N9" t="n">
-        <v>0.025167981776919</v>
+        <v>0.0251685728140791</v>
       </c>
       <c r="O9" t="n">
-        <v>17.4412772964176</v>
+        <v>17.4426106134714</v>
       </c>
       <c r="P9" t="n">
-        <v>19.0747717566163</v>
+        <v>19.0747533274448</v>
       </c>
       <c r="Q9" t="n">
-        <v>39956.2480542827</v>
+        <v>39954.5734478405</v>
       </c>
       <c r="R9" t="n">
-        <v>38670.5898664454</v>
+        <v>38670.4993985447</v>
       </c>
       <c r="S9" t="n">
-        <v>103.324640747083</v>
+        <v>103.320552020965</v>
       </c>
       <c r="T9" t="n">
-        <v>-4.03863933589642</v>
+        <v>-4.04272806201463</v>
       </c>
     </row>
     <row r="10">
@@ -5093,37 +5093,37 @@
         <v>0.026</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.0913881282996021</v>
+        <v>-0.090054811245785</v>
       </c>
       <c r="K10" t="n">
-        <v>0.684522650605378</v>
+        <v>0.684542769223703</v>
       </c>
       <c r="L10" t="n">
-        <v>2.74408984884307</v>
+        <v>2.74411006388449</v>
       </c>
       <c r="M10" t="n">
-        <v>0.026000000008817</v>
+        <v>0.0259999999952918</v>
       </c>
       <c r="N10" t="n">
-        <v>0.0252169107027416</v>
+        <v>0.0252175018065361</v>
       </c>
       <c r="O10" t="n">
-        <v>17.5516421390612</v>
+        <v>17.552975456115</v>
       </c>
       <c r="P10" t="n">
-        <v>19.0732463784814</v>
+        <v>19.073227949827</v>
       </c>
       <c r="Q10" t="n">
-        <v>39817.6577279583</v>
+        <v>39815.9837247309</v>
       </c>
       <c r="R10" t="n">
-        <v>38663.1012949494</v>
+        <v>38663.0108341294</v>
       </c>
       <c r="S10" t="n">
-        <v>102.986197160443</v>
+        <v>102.982108391786</v>
       </c>
       <c r="T10" t="n">
-        <v>-4.3770829225371</v>
+        <v>-4.38117169119441</v>
       </c>
     </row>
     <row r="11">
@@ -5155,37 +5155,37 @@
         <v>0.026</v>
       </c>
       <c r="J11" t="n">
-        <v>-0.341006535077831</v>
+        <v>-0.317923206285625</v>
       </c>
       <c r="K11" t="n">
-        <v>0.680756477697625</v>
+        <v>0.68110471768988</v>
       </c>
       <c r="L11" t="n">
-        <v>2.74030562568799</v>
+        <v>2.74065553470024</v>
       </c>
       <c r="M11" t="n">
-        <v>0.0259999999844491</v>
+        <v>0.0259999999969089</v>
       </c>
       <c r="N11" t="n">
-        <v>0.0251062596763245</v>
+        <v>0.0251164899936909</v>
       </c>
       <c r="O11" t="n">
-        <v>17.302023732283</v>
+        <v>17.3251070610752</v>
       </c>
       <c r="P11" t="n">
-        <v>19.0766961928649</v>
+        <v>19.076377205032</v>
       </c>
       <c r="Q11" t="n">
-        <v>40131.1862089296</v>
+        <v>40102.1821610345</v>
       </c>
       <c r="R11" t="n">
-        <v>38680.0402145173</v>
+        <v>38678.473559463</v>
       </c>
       <c r="S11" t="n">
-        <v>103.751666198805</v>
+        <v>103.68088104455</v>
       </c>
       <c r="T11" t="n">
-        <v>-3.61161388417453</v>
+        <v>-3.68239903843002</v>
       </c>
     </row>
     <row r="12">
@@ -5217,37 +5217,37 @@
         <v>0.026</v>
       </c>
       <c r="J12" t="n">
-        <v>-0.39343495744554</v>
+        <v>-0.370439628117808</v>
       </c>
       <c r="K12" t="n">
-        <v>0.679965559137567</v>
+        <v>0.680312455264255</v>
       </c>
       <c r="L12" t="n">
-        <v>2.73951091646933</v>
+        <v>2.73985947517528</v>
       </c>
       <c r="M12" t="n">
-        <v>0.025999999993833</v>
+        <v>0.0259999999795177</v>
       </c>
       <c r="N12" t="n">
-        <v>0.0250830258410366</v>
+        <v>0.0250932159873469</v>
       </c>
       <c r="O12" t="n">
-        <v>17.2495953099153</v>
+        <v>17.272590639243</v>
       </c>
       <c r="P12" t="n">
-        <v>19.0774206742659</v>
+        <v>19.0771029174139</v>
       </c>
       <c r="Q12" t="n">
-        <v>40197.0702416694</v>
+        <v>40168.1718420757</v>
       </c>
       <c r="R12" t="n">
-        <v>38683.5986842421</v>
+        <v>38682.0378896213</v>
       </c>
       <c r="S12" t="n">
-        <v>103.912437334957</v>
+        <v>103.841922591294</v>
       </c>
       <c r="T12" t="n">
-        <v>-3.45084274802267</v>
+        <v>-3.52135749168555</v>
       </c>
     </row>
     <row r="13">
@@ -5279,37 +5279,37 @@
         <v>0.026</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.284616104485266</v>
+        <v>-0.261422843576262</v>
       </c>
       <c r="K13" t="n">
-        <v>0.681607207302063</v>
+        <v>0.681957121290771</v>
       </c>
       <c r="L13" t="n">
-        <v>2.74116043260915</v>
+        <v>2.7415120236409</v>
       </c>
       <c r="M13" t="n">
-        <v>0.0260000000040048</v>
+        <v>0.0259999999806146</v>
       </c>
       <c r="N13" t="n">
-        <v>0.0251312519632405</v>
+        <v>0.0251415319984967</v>
       </c>
       <c r="O13" t="n">
-        <v>17.3584141628755</v>
+        <v>17.3816074237845</v>
       </c>
       <c r="P13" t="n">
-        <v>19.0759169245472</v>
+        <v>19.0755964033336</v>
       </c>
       <c r="Q13" t="n">
-        <v>40060.3358463092</v>
+        <v>40031.1990153855</v>
       </c>
       <c r="R13" t="n">
-        <v>38676.2131084794</v>
+        <v>38674.6391059965</v>
       </c>
       <c r="S13" t="n">
-        <v>103.578744211455</v>
+        <v>103.507621378628</v>
       </c>
       <c r="T13" t="n">
-        <v>-3.7845358715247</v>
+        <v>-3.85565870435232</v>
       </c>
     </row>
     <row r="14">
@@ -5341,37 +5341,37 @@
         <v>0.033</v>
       </c>
       <c r="J14" t="n">
-        <v>-0.283540256177145</v>
+        <v>-0.280963610039997</v>
       </c>
       <c r="K14" t="n">
-        <v>1.39662743424176</v>
+        <v>1.39666661716957</v>
       </c>
       <c r="L14" t="n">
-        <v>3.45960755796053</v>
+        <v>3.4596469286815</v>
       </c>
       <c r="M14" t="n">
-        <v>0.0330000000117017</v>
+        <v>0.0329999999830926</v>
       </c>
       <c r="N14" t="n">
-        <v>0.0325754763608046</v>
+        <v>0.0325766285498101</v>
       </c>
       <c r="O14" t="n">
-        <v>17.3594900111837</v>
+        <v>17.3620666573208</v>
       </c>
       <c r="P14" t="n">
-        <v>18.4209583966705</v>
+        <v>18.4209225051086</v>
       </c>
       <c r="Q14" t="n">
-        <v>39513.8980566219</v>
+        <v>39510.5846450914</v>
       </c>
       <c r="R14" t="n">
-        <v>39972.2645009952</v>
+        <v>39972.0837061798</v>
       </c>
       <c r="S14" t="n">
-        <v>98.853288773865</v>
+        <v>98.8454465759635</v>
       </c>
       <c r="T14" t="n">
-        <v>-8.50999130911495</v>
+        <v>-8.51783350701638</v>
       </c>
     </row>
     <row r="15">
@@ -5403,37 +5403,37 @@
         <v>0.033</v>
       </c>
       <c r="J15" t="n">
-        <v>-0.385280365831578</v>
+        <v>-0.38270371969443</v>
       </c>
       <c r="K15" t="n">
-        <v>1.39508028750381</v>
+        <v>1.39511946844769</v>
       </c>
       <c r="L15" t="n">
-        <v>3.45805299616704</v>
+        <v>3.45809236489456</v>
       </c>
       <c r="M15" t="n">
-        <v>0.0329999999996382</v>
+        <v>0.0329999999866624</v>
       </c>
       <c r="N15" t="n">
-        <v>0.0325299861026989</v>
+        <v>0.0325311380250382</v>
       </c>
       <c r="O15" t="n">
-        <v>17.2577499015292</v>
+        <v>17.2603265476664</v>
       </c>
       <c r="P15" t="n">
-        <v>18.4223755830824</v>
+        <v>18.4223396933378</v>
       </c>
       <c r="Q15" t="n">
-        <v>39644.7519768505</v>
+        <v>39641.4374689996</v>
       </c>
       <c r="R15" t="n">
-        <v>39979.4035623777</v>
+        <v>39979.2227469228</v>
       </c>
       <c r="S15" t="n">
-        <v>99.1629400248429</v>
+        <v>99.1550979365919</v>
       </c>
       <c r="T15" t="n">
-        <v>-8.20034005813699</v>
+        <v>-8.20818214638805</v>
       </c>
     </row>
     <row r="16">
@@ -5465,37 +5465,37 @@
         <v>0.033</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.166857854616306</v>
+        <v>-0.164281208479158</v>
       </c>
       <c r="K16" t="n">
-        <v>1.39840198010221</v>
+        <v>1.39844116829075</v>
       </c>
       <c r="L16" t="n">
-        <v>3.46139060873896</v>
+        <v>3.4614299847459</v>
       </c>
       <c r="M16" t="n">
-        <v>0.0330000000049406</v>
+        <v>0.0330000000102237</v>
       </c>
       <c r="N16" t="n">
-        <v>0.0326276584589438</v>
+        <v>0.0326288108851633</v>
       </c>
       <c r="O16" t="n">
-        <v>17.4761724127445</v>
+        <v>17.4787490588816</v>
       </c>
       <c r="P16" t="n">
-        <v>18.4193329126623</v>
+        <v>18.4192970162816</v>
       </c>
       <c r="Q16" t="n">
-        <v>39363.8791656078</v>
+        <v>39360.5670060724</v>
       </c>
       <c r="R16" t="n">
-        <v>39964.0781350212</v>
+        <v>39963.8973728804</v>
       </c>
       <c r="S16" t="n">
-        <v>98.4981538485999</v>
+        <v>98.4903114899465</v>
       </c>
       <c r="T16" t="n">
-        <v>-8.86512623438001</v>
+        <v>-8.87296859303338</v>
       </c>
     </row>
     <row r="17">
@@ -5527,37 +5527,37 @@
         <v>0.033</v>
       </c>
       <c r="J17" t="n">
-        <v>-0.757552904199768</v>
+        <v>-0.678426174659694</v>
       </c>
       <c r="K17" t="n">
-        <v>1.38942041792633</v>
+        <v>1.39062326594584</v>
       </c>
       <c r="L17" t="n">
-        <v>3.45236600036662</v>
+        <v>3.45357461331113</v>
       </c>
       <c r="M17" t="n">
-        <v>0.033000000005794</v>
+        <v>0.0329999999967665</v>
       </c>
       <c r="N17" t="n">
-        <v>0.0323636079372183</v>
+        <v>0.0323989620357821</v>
       </c>
       <c r="O17" t="n">
-        <v>16.885477363161</v>
+        <v>16.9646040927011</v>
       </c>
       <c r="P17" t="n">
-        <v>18.4275600236154</v>
+        <v>18.4264582148295</v>
       </c>
       <c r="Q17" t="n">
-        <v>40123.9219589833</v>
+        <v>40022.0256744747</v>
       </c>
       <c r="R17" t="n">
-        <v>40005.5340988797</v>
+        <v>39999.9789491081</v>
       </c>
       <c r="S17" t="n">
-        <v>100.295928707791</v>
+        <v>100.055116842423</v>
       </c>
       <c r="T17" t="n">
-        <v>-7.06735137518913</v>
+        <v>-7.30816324055688</v>
       </c>
     </row>
     <row r="18">
@@ -5589,37 +5589,37 @@
         <v>0.033</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.854986673689603</v>
+        <v>-0.776554092394349</v>
       </c>
       <c r="K18" t="n">
-        <v>1.3879393895631</v>
+        <v>1.38913158131778</v>
       </c>
       <c r="L18" t="n">
-        <v>3.45087787383533</v>
+        <v>3.4520757794424</v>
       </c>
       <c r="M18" t="n">
-        <v>0.03300000000106</v>
+        <v>0.0329999999773796</v>
       </c>
       <c r="N18" t="n">
-        <v>0.032320081334005</v>
+        <v>0.0323551188574007</v>
       </c>
       <c r="O18" t="n">
-        <v>16.7880435936712</v>
+        <v>16.8664761749664</v>
       </c>
       <c r="P18" t="n">
-        <v>18.4289166455961</v>
+        <v>18.4278245979488</v>
       </c>
       <c r="Q18" t="n">
-        <v>40249.4292790266</v>
+        <v>40148.3948390993</v>
       </c>
       <c r="R18" t="n">
-        <v>40012.3753197882</v>
+        <v>40006.8681748826</v>
       </c>
       <c r="S18" t="n">
-        <v>100.592451603645</v>
+        <v>100.353755919104</v>
       </c>
       <c r="T18" t="n">
-        <v>-6.77082847933534</v>
+        <v>-7.00952416387608</v>
       </c>
     </row>
     <row r="19">
@@ -5651,37 +5651,37 @@
         <v>0.033</v>
       </c>
       <c r="J19" t="n">
-        <v>-0.644506630947547</v>
+        <v>-0.56478195699525</v>
       </c>
       <c r="K19" t="n">
-        <v>1.39113892291695</v>
+        <v>1.39235098398685</v>
       </c>
       <c r="L19" t="n">
-        <v>3.45409274168651</v>
+        <v>3.45531061183704</v>
       </c>
       <c r="M19" t="n">
-        <v>0.0330000000329154</v>
+        <v>0.032999999986455</v>
       </c>
       <c r="N19" t="n">
-        <v>0.0324141190847596</v>
+        <v>0.0324497477140056</v>
       </c>
       <c r="O19" t="n">
-        <v>16.9985236364132</v>
+        <v>17.0782483103655</v>
       </c>
       <c r="P19" t="n">
-        <v>18.425985873044</v>
+        <v>18.424875625104</v>
       </c>
       <c r="Q19" t="n">
-        <v>39978.3534254477</v>
+        <v>39875.7248889079</v>
       </c>
       <c r="R19" t="n">
-        <v>39997.5977837826</v>
+        <v>39992.0014999253</v>
       </c>
       <c r="S19" t="n">
-        <v>99.9518862146699</v>
+        <v>99.7092503334258</v>
       </c>
       <c r="T19" t="n">
-        <v>-7.41139386831006</v>
+        <v>-7.65402974955407</v>
       </c>
     </row>
     <row r="20">
@@ -5713,37 +5713,37 @@
         <v>0.02</v>
       </c>
       <c r="J20" t="n">
-        <v>-0.0254857052549629</v>
+        <v>-0.0252593550460228</v>
       </c>
       <c r="K20" t="n">
-        <v>0.07282989908791</v>
+        <v>0.0728332912016984</v>
       </c>
       <c r="L20" t="n">
-        <v>2.12946541953578</v>
+        <v>2.12946882790703</v>
       </c>
       <c r="M20" t="n">
-        <v>0.0199999999856091</v>
+        <v>0.0199999999939684</v>
       </c>
       <c r="N20" t="n">
-        <v>0.0188705028858045</v>
+        <v>0.0188706025711718</v>
       </c>
       <c r="O20" t="n">
-        <v>17.6175445621058</v>
+        <v>17.6177709123148</v>
       </c>
       <c r="P20" t="n">
-        <v>19.6335569388714</v>
+        <v>19.6335538316952</v>
       </c>
       <c r="Q20" t="n">
-        <v>40181.7693932306</v>
+        <v>40181.4908991144</v>
       </c>
       <c r="R20" t="n">
-        <v>37574.6852115126</v>
+        <v>37574.6702876911</v>
       </c>
       <c r="S20" t="n">
-        <v>106.938405916224</v>
+        <v>106.937707214632</v>
       </c>
       <c r="T20" t="n">
-        <v>-0.424874166756325</v>
+        <v>-0.425572868347814</v>
       </c>
     </row>
     <row r="21">
@@ -5775,37 +5775,37 @@
         <v>0.02</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.0346378988383578</v>
+        <v>-0.0344115486294178</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0726927356922062</v>
+        <v>0.0726961274288146</v>
       </c>
       <c r="L21" t="n">
-        <v>2.12932759875306</v>
+        <v>2.12933100674533</v>
       </c>
       <c r="M21" t="n">
-        <v>0.0200000000002583</v>
+        <v>0.0199999999845193</v>
       </c>
       <c r="N21" t="n">
-        <v>0.0188664753834344</v>
+        <v>0.0188665749670807</v>
       </c>
       <c r="O21" t="n">
-        <v>17.6083923685224</v>
+        <v>17.6086187187314</v>
       </c>
       <c r="P21" t="n">
-        <v>19.6336825805419</v>
+        <v>19.6336794737111</v>
       </c>
       <c r="Q21" t="n">
-        <v>40193.0299894161</v>
+        <v>40192.7514957645</v>
       </c>
       <c r="R21" t="n">
-        <v>37575.2885179576</v>
+        <v>37575.2735990816</v>
       </c>
       <c r="S21" t="n">
-        <v>106.966657009719</v>
+        <v>106.965958317725</v>
       </c>
       <c r="T21" t="n">
-        <v>-0.396623073260784</v>
+        <v>-0.397321765255398</v>
       </c>
     </row>
     <row r="22">
@@ -5837,37 +5837,37 @@
         <v>0.02</v>
       </c>
       <c r="J22" t="n">
-        <v>-0.0162341236259994</v>
+        <v>-0.0160077734170594</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0729685533773562</v>
+        <v>0.0729719461486873</v>
       </c>
       <c r="L22" t="n">
-        <v>2.1296047383577</v>
+        <v>2.12960814738965</v>
       </c>
       <c r="M22" t="n">
-        <v>0.0199999999946143</v>
+        <v>0.0200000000009677</v>
       </c>
       <c r="N22" t="n">
-        <v>0.0188745743566012</v>
+        <v>0.0188746739586174</v>
       </c>
       <c r="O22" t="n">
-        <v>17.6267961437348</v>
+        <v>17.6270224939437</v>
       </c>
       <c r="P22" t="n">
-        <v>19.6334299315423</v>
+        <v>19.6334268237637</v>
       </c>
       <c r="Q22" t="n">
-        <v>40170.3868449224</v>
+        <v>40170.1083594683</v>
       </c>
       <c r="R22" t="n">
-        <v>37574.0753540371</v>
+        <v>37574.0604308289</v>
       </c>
       <c r="S22" t="n">
-        <v>106.909847990727</v>
+        <v>106.909149287761</v>
       </c>
       <c r="T22" t="n">
-        <v>-0.453432092252598</v>
+        <v>-0.454130795219257</v>
       </c>
     </row>
     <row r="23">
@@ -5899,37 +5899,37 @@
         <v>0.02</v>
       </c>
       <c r="J23" t="n">
-        <v>-0.0822707695848912</v>
+        <v>-0.0823070036456097</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0719788820351838</v>
+        <v>0.071978338639114</v>
       </c>
       <c r="L23" t="n">
-        <v>2.12861032378866</v>
+        <v>2.12860977778824</v>
       </c>
       <c r="M23" t="n">
-        <v>0.0199999999895371</v>
+        <v>0.0200000000031326</v>
       </c>
       <c r="N23" t="n">
-        <v>0.0188455148203448</v>
+        <v>0.0188454989168403</v>
       </c>
       <c r="O23" t="n">
-        <v>17.5607594977759</v>
+        <v>17.5607232637152</v>
       </c>
       <c r="P23" t="n">
-        <v>19.6343364704917</v>
+        <v>19.6343369682425</v>
       </c>
       <c r="Q23" t="n">
-        <v>40251.6415476907</v>
+        <v>40251.6861354858</v>
       </c>
       <c r="R23" t="n">
-        <v>37578.4285916403</v>
+        <v>37578.4309795631</v>
       </c>
       <c r="S23" t="n">
-        <v>107.113690104235</v>
+        <v>107.113801950317</v>
       </c>
       <c r="T23" t="n">
-        <v>-0.249589978745206</v>
+        <v>-0.249478132663015</v>
       </c>
     </row>
     <row r="24">
@@ -5961,37 +5961,37 @@
         <v>0.02</v>
       </c>
       <c r="J24" t="n">
-        <v>-0.0913934496556274</v>
+        <v>-0.0914296837163459</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0718421678274633</v>
+        <v>0.0718416241189225</v>
       </c>
       <c r="L24" t="n">
-        <v>2.12847295434675</v>
+        <v>2.12847240803236</v>
       </c>
       <c r="M24" t="n">
-        <v>0.0199999999835945</v>
+        <v>0.0199999999925828</v>
       </c>
       <c r="N24" t="n">
-        <v>0.0188415006548048</v>
+        <v>0.0188414846906613</v>
       </c>
       <c r="O24" t="n">
-        <v>17.5516368177052</v>
+        <v>17.5516005836445</v>
       </c>
       <c r="P24" t="n">
-        <v>19.634461700706</v>
+        <v>19.634462198743</v>
       </c>
       <c r="Q24" t="n">
-        <v>40262.867909424</v>
+        <v>40262.9124978303</v>
       </c>
       <c r="R24" t="n">
-        <v>37579.0300044955</v>
+        <v>37579.0323915506</v>
       </c>
       <c r="S24" t="n">
-        <v>107.141849868417</v>
+        <v>107.141961715021</v>
       </c>
       <c r="T24" t="n">
-        <v>-0.221430214562915</v>
+        <v>-0.22131836795927</v>
       </c>
     </row>
     <row r="25">
@@ -6023,37 +6023,37 @@
         <v>0.02</v>
       </c>
       <c r="J25" t="n">
-        <v>-0.0730537432937967</v>
+        <v>-0.0730899773545152</v>
       </c>
       <c r="K25" t="n">
-        <v>0.0721170116787752</v>
+        <v>0.0721164671411194</v>
       </c>
       <c r="L25" t="n">
-        <v>2.12874911545025</v>
+        <v>2.12874856830276</v>
       </c>
       <c r="M25" t="n">
-        <v>0.0200000000202882</v>
+        <v>0.0200000000002025</v>
       </c>
       <c r="N25" t="n">
-        <v>0.0188495706886871</v>
+        <v>0.0188495547058967</v>
       </c>
       <c r="O25" t="n">
-        <v>17.569976524067</v>
+        <v>17.5699402900063</v>
       </c>
       <c r="P25" t="n">
-        <v>19.6342099437382</v>
+        <v>19.6342104425347</v>
       </c>
       <c r="Q25" t="n">
-        <v>40240.2994200197</v>
+        <v>40240.3440093889</v>
       </c>
       <c r="R25" t="n">
-        <v>37577.8209683877</v>
+        <v>37577.8233558097</v>
       </c>
       <c r="S25" t="n">
-        <v>107.085239066607</v>
+        <v>107.085350921922</v>
       </c>
       <c r="T25" t="n">
-        <v>-0.278041016372569</v>
+        <v>-0.277929161057557</v>
       </c>
     </row>
   </sheetData>
@@ -6070,7 +6070,7 @@
     <col min="1" max="1" width="46.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="46.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="21.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="22.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="21.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6367,7 +6367,7 @@
         <v>101</v>
       </c>
       <c r="B7" t="n">
-        <v>8.16574765183793</v>
+        <v>8.01534691145987</v>
       </c>
     </row>
     <row r="8">
@@ -6375,7 +6375,7 @@
         <v>102</v>
       </c>
       <c r="B8" t="n">
-        <v>4.73452914373081</v>
+        <v>4.58412840335275</v>
       </c>
     </row>
     <row r="9">
@@ -6383,7 +6383,7 @@
         <v>103</v>
       </c>
       <c r="B9" t="n">
-        <v>11.6324516198077</v>
+        <v>11.4820508794297</v>
       </c>
     </row>
     <row r="10">
@@ -6391,7 +6391,7 @@
         <v>104</v>
       </c>
       <c r="B10" t="n">
-        <v>105.153773547655</v>
+        <v>113.264608019879</v>
       </c>
     </row>
     <row r="11">
@@ -6399,7 +6399,7 @@
         <v>105</v>
       </c>
       <c r="B11" t="n">
-        <v>84.8475732441497</v>
+        <v>92.9243243953035</v>
       </c>
     </row>
     <row r="12">
@@ -6407,7 +6407,7 @@
         <v>106</v>
       </c>
       <c r="B12" t="n">
-        <v>126.994510443822</v>
+        <v>135.147923034591</v>
       </c>
     </row>
     <row r="13">
@@ -6415,7 +6415,7 @@
         <v>107</v>
       </c>
       <c r="B13" t="n">
-        <v>170.746253043999</v>
+        <v>200.79414919708</v>
       </c>
     </row>
     <row r="14">
@@ -6423,7 +6423,7 @@
         <v>108</v>
       </c>
       <c r="B14" t="n">
-        <v>131.703881974806</v>
+        <v>161.473628226743</v>
       </c>
     </row>
     <row r="15">
@@ -6431,7 +6431,7 @@
         <v>109</v>
       </c>
       <c r="B15" t="n">
-        <v>216.044660068707</v>
+        <v>246.332156595892</v>
       </c>
     </row>
   </sheetData>
@@ -6488,7 +6488,7 @@
         <v>114</v>
       </c>
       <c r="C7" t="n">
-        <v>15.7351498494936</v>
+        <v>30.0077025141354</v>
       </c>
       <c r="D7" t="s">
         <v>115</v>
@@ -6502,7 +6502,7 @@
         <v>114</v>
       </c>
       <c r="C8" t="n">
-        <v>-4.5266729135019</v>
+        <v>9.71167065833561</v>
       </c>
       <c r="D8" t="s">
         <v>115</v>
@@ -6516,7 +6516,7 @@
         <v>114</v>
       </c>
       <c r="C9" t="n">
-        <v>37.5102889930149</v>
+        <v>51.8252224882954</v>
       </c>
       <c r="D9" t="s">
         <v>115</v>
@@ -6530,7 +6530,7 @@
         <v>114</v>
       </c>
       <c r="C10" t="n">
-        <v>-36.0319710124613</v>
+        <v>15.6102845632649</v>
       </c>
       <c r="D10" t="s">
         <v>115</v>
@@ -6544,7 +6544,7 @@
         <v>114</v>
       </c>
       <c r="C11" t="n">
-        <v>-74.7252766878519</v>
+        <v>-23.385412749124</v>
       </c>
       <c r="D11" t="s">
         <v>115</v>
@@ -6558,7 +6558,7 @@
         <v>114</v>
       </c>
       <c r="C12" t="n">
-        <v>9.02976474219577</v>
+        <v>60.9230398695281</v>
       </c>
       <c r="D12" t="s">
         <v>115</v>
@@ -6614,7 +6614,7 @@
         <v>116</v>
       </c>
       <c r="C16" t="n">
-        <v>52.7340772104844</v>
+        <v>49.4313684315475</v>
       </c>
       <c r="D16" t="s">
         <v>117</v>
@@ -6628,7 +6628,7 @@
         <v>116</v>
       </c>
       <c r="C17" t="n">
-        <v>52.7340772104844</v>
+        <v>49.4313684315475</v>
       </c>
       <c r="D17" t="s">
         <v>117</v>
@@ -6642,7 +6642,7 @@
         <v>116</v>
       </c>
       <c r="C18" t="n">
-        <v>52.7340772104844</v>
+        <v>49.4313684315475</v>
       </c>
       <c r="D18" t="s">
         <v>117</v>
@@ -6656,7 +6656,7 @@
         <v>116</v>
       </c>
       <c r="C19" t="n">
-        <v>122.932200326053</v>
+        <v>110.676210036276</v>
       </c>
       <c r="D19" t="s">
         <v>117</v>
@@ -6670,7 +6670,7 @@
         <v>116</v>
       </c>
       <c r="C20" t="n">
-        <v>122.932200326053</v>
+        <v>110.676210036276</v>
       </c>
       <c r="D20" t="s">
         <v>117</v>
@@ -6684,7 +6684,7 @@
         <v>116</v>
       </c>
       <c r="C21" t="n">
-        <v>122.932200326053</v>
+        <v>110.676210036276</v>
       </c>
       <c r="D21" t="s">
         <v>117</v>
@@ -6740,7 +6740,7 @@
         <v>118</v>
       </c>
       <c r="C25" t="n">
-        <v>0.0257895279983131</v>
+        <v>0.0480621953411173</v>
       </c>
       <c r="D25" t="s">
         <v>119</v>
@@ -6754,7 +6754,7 @@
         <v>118</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.0185880125118274</v>
+        <v>0.0038104265659058</v>
       </c>
       <c r="D26" t="s">
         <v>119</v>
@@ -6768,7 +6768,7 @@
         <v>118</v>
       </c>
       <c r="C27" t="n">
-        <v>0.091387280644085</v>
+        <v>0.113857235893192</v>
       </c>
       <c r="D27" t="s">
         <v>119</v>
@@ -6782,7 +6782,7 @@
         <v>118</v>
       </c>
       <c r="C28" t="n">
-        <v>-0.155147368337566</v>
+        <v>0.063487409624031</v>
       </c>
       <c r="D28" t="s">
         <v>119</v>
@@ -6796,7 +6796,7 @@
         <v>118</v>
       </c>
       <c r="C29" t="n">
-        <v>-0.504212762140014</v>
+        <v>-0.261336248324369</v>
       </c>
       <c r="D29" t="s">
         <v>119</v>
@@ -6810,7 +6810,7 @@
         <v>118</v>
       </c>
       <c r="C30" t="n">
-        <v>0.0815239017138083</v>
+        <v>0.288739502173485</v>
       </c>
       <c r="D30" t="s">
         <v>119</v>
@@ -6866,7 +6866,7 @@
         <v>120</v>
       </c>
       <c r="C34" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="D34" t="s">
         <v>121</v>
@@ -6880,7 +6880,7 @@
         <v>120</v>
       </c>
       <c r="C35" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="D35" t="s">
         <v>121</v>
@@ -6894,7 +6894,7 @@
         <v>120</v>
       </c>
       <c r="C36" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="D36" t="s">
         <v>121</v>
@@ -6908,7 +6908,7 @@
         <v>120</v>
       </c>
       <c r="C37" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="D37" t="s">
         <v>121</v>
@@ -6922,7 +6922,7 @@
         <v>120</v>
       </c>
       <c r="C38" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="D38" t="s">
         <v>121</v>
@@ -6936,7 +6936,7 @@
         <v>120</v>
       </c>
       <c r="C39" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="D39" t="s">
         <v>121</v>
@@ -6950,7 +6950,7 @@
         <v>120</v>
       </c>
       <c r="C40" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="D40" t="s">
         <v>121</v>
@@ -6964,7 +6964,7 @@
         <v>120</v>
       </c>
       <c r="C41" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="D41" t="s">
         <v>121</v>
@@ -6978,7 +6978,7 @@
         <v>120</v>
       </c>
       <c r="C42" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="D42" t="s">
         <v>121</v>
@@ -7052,10 +7052,10 @@
       <c r="C7"/>
       <c r="D7"/>
       <c r="E7" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="F7" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G7" t="s">
         <v>121</v>
@@ -7078,7 +7078,7 @@
         <v>-0.368722591245188</v>
       </c>
       <c r="F8" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G8" t="s">
         <v>131</v>
@@ -7101,7 +7101,7 @@
         <v>3.93546001088544</v>
       </c>
       <c r="F9" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G9" t="s">
         <v>133</v>
@@ -7124,7 +7124,7 @@
         <v>-3.7673125102699</v>
       </c>
       <c r="F10" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G10" t="s">
         <v>135</v>
@@ -7140,10 +7140,10 @@
       <c r="C11"/>
       <c r="D11"/>
       <c r="E11" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="F11" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G11" t="s">
         <v>121</v>
@@ -7166,7 +7166,7 @@
         <v>0.717580226326447</v>
       </c>
       <c r="F12" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G12" t="s">
         <v>131</v>
@@ -7189,7 +7189,7 @@
         <v>-4.72220153060562</v>
       </c>
       <c r="F13" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G13" t="s">
         <v>133</v>
@@ -7212,7 +7212,7 @@
         <v>0.372827705542704</v>
       </c>
       <c r="F14" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G14" t="s">
         <v>135</v>
@@ -7228,10 +7228,10 @@
       <c r="C15"/>
       <c r="D15"/>
       <c r="E15" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="F15" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G15" t="s">
         <v>121</v>
@@ -7254,7 +7254,7 @@
         <v>-1.45311266812115</v>
       </c>
       <c r="F16" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G16" t="s">
         <v>131</v>
@@ -7277,7 +7277,7 @@
         <v>12.6572121884519</v>
       </c>
       <c r="F17" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G17" t="s">
         <v>133</v>
@@ -7300,7 +7300,7 @@
         <v>-7.93797064299088</v>
       </c>
       <c r="F18" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="G18" t="s">
         <v>135</v>
@@ -7316,10 +7316,10 @@
       <c r="C19"/>
       <c r="D19"/>
       <c r="E19" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="F19" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G19" t="s">
         <v>121</v>
@@ -7336,13 +7336,13 @@
         <v>-100.96774507013</v>
       </c>
       <c r="D20" t="n">
-        <v>-100.344407038839</v>
+        <v>-99.8892532720676</v>
       </c>
       <c r="E20" t="n">
-        <v>0.623338031290842</v>
+        <v>1.07849179806213</v>
       </c>
       <c r="F20" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G20" t="s">
         <v>131</v>
@@ -7359,13 +7359,13 @@
         <v>3010.43359034049</v>
       </c>
       <c r="D21" t="n">
-        <v>3073.39510856483</v>
+        <v>3079.4865976585</v>
       </c>
       <c r="E21" t="n">
-        <v>62.9615182243424</v>
+        <v>69.0530073180144</v>
       </c>
       <c r="F21" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G21" t="s">
         <v>133</v>
@@ -7382,13 +7382,13 @@
         <v>1970.92352019412</v>
       </c>
       <c r="D22" t="n">
-        <v>1975.83368052646</v>
+        <v>1980.27915421907</v>
       </c>
       <c r="E22" t="n">
-        <v>4.91016033234359</v>
+        <v>9.3556340249479</v>
       </c>
       <c r="F22" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G22" t="s">
         <v>135</v>
@@ -7404,10 +7404,10 @@
       <c r="C23"/>
       <c r="D23"/>
       <c r="E23" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="F23" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G23" t="s">
         <v>121</v>
@@ -7424,13 +7424,13 @@
         <v>-100.96774507013</v>
       </c>
       <c r="D24" t="n">
-        <v>-93.6888221250927</v>
+        <v>-93.2193727258138</v>
       </c>
       <c r="E24" t="n">
-        <v>7.27892294503704</v>
+        <v>7.74837234431591</v>
       </c>
       <c r="F24" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G24" t="s">
         <v>131</v>
@@ -7447,13 +7447,13 @@
         <v>3010.43359034049</v>
       </c>
       <c r="D25" t="n">
-        <v>3021.5554073223</v>
+        <v>3027.49767610528</v>
       </c>
       <c r="E25" t="n">
-        <v>11.121816981813</v>
+        <v>17.064085764795</v>
       </c>
       <c r="F25" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G25" t="s">
         <v>133</v>
@@ -7470,13 +7470,13 @@
         <v>1970.92352019412</v>
       </c>
       <c r="D26" t="n">
-        <v>2000.71159655174</v>
+        <v>2005.25791160146</v>
       </c>
       <c r="E26" t="n">
-        <v>29.7880763576211</v>
+        <v>34.3343914073391</v>
       </c>
       <c r="F26" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G26" t="s">
         <v>135</v>
@@ -7492,10 +7492,10 @@
       <c r="C27"/>
       <c r="D27"/>
       <c r="E27" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="F27" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G27" t="s">
         <v>121</v>
@@ -7512,13 +7512,13 @@
         <v>-100.96774507013</v>
       </c>
       <c r="D28" t="n">
-        <v>-106.858683756629</v>
+        <v>-106.418859519679</v>
       </c>
       <c r="E28" t="n">
-        <v>-5.89093868649896</v>
+        <v>-5.45111444954932</v>
       </c>
       <c r="F28" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G28" t="s">
         <v>131</v>
@@ -7535,13 +7535,13 @@
         <v>3010.43359034049</v>
       </c>
       <c r="D29" t="n">
-        <v>3127.66863442254</v>
+        <v>3133.91702913126</v>
       </c>
       <c r="E29" t="n">
-        <v>117.235044082048</v>
+        <v>123.483438790769</v>
       </c>
       <c r="F29" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G29" t="s">
         <v>133</v>
@@ -7558,13 +7558,13 @@
         <v>1970.92352019412</v>
       </c>
       <c r="D30" t="n">
-        <v>1949.91516828272</v>
+        <v>1954.26164400864</v>
       </c>
       <c r="E30" t="n">
-        <v>-21.0083519114044</v>
+        <v>-16.6618761854836</v>
       </c>
       <c r="F30" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="G30" t="s">
         <v>135</v>
@@ -7580,10 +7580,10 @@
       <c r="C31"/>
       <c r="D31"/>
       <c r="E31" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="F31" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G31" t="s">
         <v>121</v>
@@ -7600,13 +7600,13 @@
         <v>-100.96774507013</v>
       </c>
       <c r="D32" t="n">
-        <v>-101.895654142962</v>
+        <v>-100.229912849212</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.927909072832591</v>
+        <v>0.737832220917753</v>
       </c>
       <c r="F32" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G32" t="s">
         <v>131</v>
@@ -7623,13 +7623,13 @@
         <v>3010.43359034049</v>
       </c>
       <c r="D33" t="n">
-        <v>3109.39525163244</v>
+        <v>3131.17450717651</v>
       </c>
       <c r="E33" t="n">
-        <v>98.9616612919495</v>
+        <v>120.740916836021</v>
       </c>
       <c r="F33" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G33" t="s">
         <v>133</v>
@@ -7646,13 +7646,13 @@
         <v>1970.92352019412</v>
       </c>
       <c r="D34" t="n">
-        <v>1959.63484992026</v>
+        <v>1975.79475314635</v>
       </c>
       <c r="E34" t="n">
-        <v>-11.2886702738613</v>
+        <v>4.87123295222636</v>
       </c>
       <c r="F34" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G34" t="s">
         <v>135</v>
@@ -7668,10 +7668,10 @@
       <c r="C35"/>
       <c r="D35"/>
       <c r="E35" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="F35" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G35" t="s">
         <v>121</v>
@@ -7688,13 +7688,13 @@
         <v>-100.96774507013</v>
       </c>
       <c r="D36" t="n">
-        <v>-88.5670719690749</v>
+        <v>-86.8208685103625</v>
       </c>
       <c r="E36" t="n">
-        <v>12.4006731010548</v>
+        <v>14.1468765597672</v>
       </c>
       <c r="F36" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G36" t="s">
         <v>131</v>
@@ -7711,13 +7711,13 @@
         <v>3010.43359034049</v>
       </c>
       <c r="D37" t="n">
-        <v>3009.05463444814</v>
+        <v>3029.7503330047</v>
       </c>
       <c r="E37" t="n">
-        <v>-1.37895589235222</v>
+        <v>19.3167426642071</v>
       </c>
       <c r="F37" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G37" t="s">
         <v>133</v>
@@ -7734,13 +7734,13 @@
         <v>1970.92352019412</v>
       </c>
       <c r="D38" t="n">
-        <v>2007.60451386148</v>
+        <v>2024.48936200897</v>
       </c>
       <c r="E38" t="n">
-        <v>36.6809936673592</v>
+        <v>53.5658418148544</v>
       </c>
       <c r="F38" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G38" t="s">
         <v>135</v>
@@ -7756,10 +7756,10 @@
       <c r="C39"/>
       <c r="D39"/>
       <c r="E39" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="F39" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G39" t="s">
         <v>121</v>
@@ -7776,13 +7776,13 @@
         <v>-100.96774507013</v>
       </c>
       <c r="D40" t="n">
-        <v>-114.468920469056</v>
+        <v>-112.964773527375</v>
       </c>
       <c r="E40" t="n">
-        <v>-13.5011753989266</v>
+        <v>-11.9970284572449</v>
       </c>
       <c r="F40" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G40" t="s">
         <v>131</v>
@@ -7799,13 +7799,13 @@
         <v>3010.43359034049</v>
       </c>
       <c r="D41" t="n">
-        <v>3219.40250129783</v>
+        <v>3242.30436050558</v>
       </c>
       <c r="E41" t="n">
-        <v>208.968910957338</v>
+        <v>231.870770165091</v>
       </c>
       <c r="F41" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G41" t="s">
         <v>133</v>
@@ -7822,13 +7822,13 @@
         <v>1970.92352019412</v>
       </c>
       <c r="D42" t="n">
-        <v>1907.49927360567</v>
+        <v>1922.93776789425</v>
       </c>
       <c r="E42" t="n">
-        <v>-63.4242465884479</v>
+        <v>-47.985752299868</v>
       </c>
       <c r="F42" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="G42" t="s">
         <v>135</v>
@@ -7889,16 +7889,16 @@
         <v>104</v>
       </c>
       <c r="B7" t="n">
-        <v>68.4950165879764</v>
+        <v>79.4871331410241</v>
       </c>
       <c r="C7" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="D7" t="n">
-        <v>105.153773547655</v>
+        <v>113.264608019879</v>
       </c>
       <c r="E7" t="n">
-        <v>404.350262630913</v>
+        <v>441.530599436801</v>
       </c>
     </row>
     <row r="8">
@@ -7906,16 +7906,16 @@
         <v>105</v>
       </c>
       <c r="B8" t="n">
-        <v>48.1888162844707</v>
+        <v>59.146849516449</v>
       </c>
       <c r="C8" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="D8" t="n">
-        <v>84.8475732441497</v>
+        <v>92.9243243953035</v>
       </c>
       <c r="E8" t="n">
-        <v>404.350262630913</v>
+        <v>441.530599436801</v>
       </c>
     </row>
     <row r="9">
@@ -7923,16 +7923,16 @@
         <v>106</v>
       </c>
       <c r="B9" t="n">
-        <v>90.3357534841434</v>
+        <v>101.370448155736</v>
       </c>
       <c r="C9" t="n">
-        <v>36.658756959679</v>
+        <v>33.7774748788545</v>
       </c>
       <c r="D9" t="n">
-        <v>126.994510443822</v>
+        <v>135.147923034591</v>
       </c>
       <c r="E9" t="n">
-        <v>404.350262630913</v>
+        <v>441.530599436801</v>
       </c>
     </row>
     <row r="10">
@@ -7940,16 +7940,16 @@
         <v>107</v>
       </c>
       <c r="B10" t="n">
-        <v>86.7450819452543</v>
+        <v>126.349982009165</v>
       </c>
       <c r="C10" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="D10" t="n">
-        <v>170.746253043999</v>
+        <v>200.79414919708</v>
       </c>
       <c r="E10" t="n">
-        <v>632.501080833316</v>
+        <v>767.132420609509</v>
       </c>
     </row>
     <row r="11">
@@ -7957,16 +7957,16 @@
         <v>108</v>
       </c>
       <c r="B11" t="n">
-        <v>47.7027108760613</v>
+        <v>87.0294610388273</v>
       </c>
       <c r="C11" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="D11" t="n">
-        <v>131.703881974806</v>
+        <v>161.473628226743</v>
       </c>
       <c r="E11" t="n">
-        <v>632.501080833316</v>
+        <v>767.132420609509</v>
       </c>
     </row>
     <row r="12">
@@ -7974,16 +7974,16 @@
         <v>109</v>
       </c>
       <c r="B12" t="n">
-        <v>132.043488969963</v>
+        <v>171.887989407977</v>
       </c>
       <c r="C12" t="n">
-        <v>84.0011710987443</v>
+        <v>74.4441671879153</v>
       </c>
       <c r="D12" t="n">
-        <v>216.044660068707</v>
+        <v>246.332156595892</v>
       </c>
       <c r="E12" t="n">
-        <v>632.501080833316</v>
+        <v>767.132420609509</v>
       </c>
     </row>
     <row r="13">
@@ -7994,10 +7994,10 @@
         <v>-0.200575090630082</v>
       </c>
       <c r="C13" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="D13" t="n">
-        <v>8.16574765183793</v>
+        <v>8.01534691145987</v>
       </c>
       <c r="E13" t="n">
         <v>28.4967461669469</v>
@@ -8011,10 +8011,10 @@
         <v>-3.6317935987372</v>
       </c>
       <c r="C14" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="D14" t="n">
-        <v>4.73452914373081</v>
+        <v>4.58412840335275</v>
       </c>
       <c r="E14" t="n">
         <v>28.4967461669469</v>
@@ -8028,10 +8028,10 @@
         <v>3.26612887733972</v>
       </c>
       <c r="C15" t="n">
-        <v>8.36632274246801</v>
+        <v>8.21592200208995</v>
       </c>
       <c r="D15" t="n">
-        <v>11.6324516198077</v>
+        <v>11.4820508794297</v>
       </c>
       <c r="E15" t="n">
         <v>28.4967461669469</v>
@@ -8080,7 +8080,7 @@
         <v>101</v>
       </c>
       <c r="B7" t="n">
-        <v>8.16574765183793</v>
+        <v>8.01534691145987</v>
       </c>
     </row>
     <row r="8">
@@ -8088,7 +8088,7 @@
         <v>102</v>
       </c>
       <c r="B8" t="n">
-        <v>4.73452914373081</v>
+        <v>4.58412840335275</v>
       </c>
     </row>
     <row r="9">
@@ -8096,7 +8096,7 @@
         <v>103</v>
       </c>
       <c r="B9" t="n">
-        <v>11.6324516198077</v>
+        <v>11.4820508794297</v>
       </c>
     </row>
     <row r="10">
@@ -8104,7 +8104,7 @@
         <v>141</v>
       </c>
       <c r="B10" t="n">
-        <v>29.5237216465691</v>
+        <v>29.4720839888619</v>
       </c>
     </row>
     <row r="11">
@@ -8112,7 +8112,7 @@
         <v>142</v>
       </c>
       <c r="B11" t="n">
-        <v>26.0814025287624</v>
+        <v>26.0297648710552</v>
       </c>
     </row>
     <row r="12">
@@ -8120,7 +8120,7 @@
         <v>143</v>
       </c>
       <c r="B12" t="n">
-        <v>33.0034225533761</v>
+        <v>32.9517848956689</v>
       </c>
     </row>
     <row r="13">
@@ -8128,7 +8128,7 @@
         <v>104</v>
       </c>
       <c r="B13" t="n">
-        <v>105.153773547655</v>
+        <v>113.264608019879</v>
       </c>
     </row>
     <row r="14">
@@ -8136,7 +8136,7 @@
         <v>105</v>
       </c>
       <c r="B14" t="n">
-        <v>84.8475732441497</v>
+        <v>92.9243243953035</v>
       </c>
     </row>
     <row r="15">
@@ -8144,7 +8144,7 @@
         <v>106</v>
       </c>
       <c r="B15" t="n">
-        <v>126.994510443822</v>
+        <v>135.147923034591</v>
       </c>
     </row>
     <row r="16">
@@ -8152,7 +8152,7 @@
         <v>144</v>
       </c>
       <c r="B16" t="n">
-        <v>179.691439362169</v>
+        <v>179.378215374913</v>
       </c>
     </row>
     <row r="17">
@@ -8160,7 +8160,7 @@
         <v>145</v>
       </c>
       <c r="B17" t="n">
-        <v>159.088464667368</v>
+        <v>158.775240680112</v>
       </c>
     </row>
     <row r="18">
@@ -8168,7 +8168,7 @@
         <v>146</v>
       </c>
       <c r="B18" t="n">
-        <v>201.834183496512</v>
+        <v>201.520959509256</v>
       </c>
     </row>
     <row r="19">
@@ -8176,7 +8176,7 @@
         <v>107</v>
       </c>
       <c r="B19" t="n">
-        <v>170.746253043999</v>
+        <v>200.79414919708</v>
       </c>
     </row>
     <row r="20">
@@ -8184,7 +8184,7 @@
         <v>108</v>
       </c>
       <c r="B20" t="n">
-        <v>131.703881974806</v>
+        <v>161.473628226743</v>
       </c>
     </row>
     <row r="21">
@@ -8192,7 +8192,7 @@
         <v>109</v>
       </c>
       <c r="B21" t="n">
-        <v>216.044660068707</v>
+        <v>246.332156595892</v>
       </c>
     </row>
     <row r="22">
@@ -8200,7 +8200,7 @@
         <v>147</v>
       </c>
       <c r="B22" t="n">
-        <v>360.686330211178</v>
+        <v>360.060089694361</v>
       </c>
     </row>
     <row r="23">
@@ -8208,7 +8208,7 @@
         <v>148</v>
       </c>
       <c r="B23" t="n">
-        <v>319.91837948376</v>
+        <v>319.292138966943</v>
       </c>
     </row>
     <row r="24">
@@ -8216,7 +8216,7 @@
         <v>149</v>
       </c>
       <c r="B24" t="n">
-        <v>407.441758466034</v>
+        <v>406.815517949216</v>
       </c>
     </row>
   </sheetData>
@@ -8280,10 +8280,10 @@
         <v>0.554723007083343</v>
       </c>
       <c r="D7" t="n">
-        <v>0.557044523203491</v>
+        <v>0.556846975499188</v>
       </c>
       <c r="E7" t="n">
-        <v>0.00232151612014808</v>
+        <v>0.00212396841584506</v>
       </c>
     </row>
     <row r="8">
@@ -8297,10 +8297,10 @@
         <v>0.591605525530161</v>
       </c>
       <c r="D8" t="n">
-        <v>0.593927531176733</v>
+        <v>0.593727708415495</v>
       </c>
       <c r="E8" t="n">
-        <v>0.00232200564657226</v>
+        <v>0.00212218288533417</v>
       </c>
     </row>
     <row r="9">
@@ -8314,10 +8314,10 @@
         <v>0.554723007083343</v>
       </c>
       <c r="D9" t="n">
-        <v>0.546523309255003</v>
+        <v>0.546302636014886</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.00819969782833963</v>
+        <v>-0.0084203710684565</v>
       </c>
     </row>
     <row r="10">
@@ -8331,10 +8331,10 @@
         <v>0.591605525530161</v>
       </c>
       <c r="D10" t="n">
-        <v>0.582265110624254</v>
+        <v>0.58204777395084</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.00934041490590731</v>
+        <v>-0.00955775157932159</v>
       </c>
     </row>
     <row r="11">
@@ -8348,10 +8348,10 @@
         <v>0.554723007083343</v>
       </c>
       <c r="D11" t="n">
-        <v>0.56762009222294</v>
+        <v>0.567436925514403</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0128970851395976</v>
+        <v>0.0127139184310602</v>
       </c>
     </row>
     <row r="12">
@@ -8365,10 +8365,10 @@
         <v>0.591605525530161</v>
       </c>
       <c r="D12" t="n">
-        <v>0.605597422990439</v>
+        <v>0.60542710730706</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0139918974602777</v>
+        <v>0.0138215817768991</v>
       </c>
     </row>
     <row r="13">
@@ -8382,10 +8382,10 @@
         <v>0.554723007083343</v>
       </c>
       <c r="D13" t="n">
-        <v>0.560442568525692</v>
+        <v>0.559636303883901</v>
       </c>
       <c r="E13" t="n">
-        <v>0.00571956144234964</v>
+        <v>0.00491329680055819</v>
       </c>
     </row>
     <row r="14">
@@ -8399,10 +8399,10 @@
         <v>0.591605525530161</v>
       </c>
       <c r="D14" t="n">
-        <v>0.597351561735813</v>
+        <v>0.596550196912608</v>
       </c>
       <c r="E14" t="n">
-        <v>0.00574603620565162</v>
+        <v>0.00494467138244681</v>
       </c>
     </row>
     <row r="15">
@@ -8416,10 +8416,10 @@
         <v>0.554723007083343</v>
       </c>
       <c r="D15" t="n">
-        <v>0.539796815332324</v>
+        <v>0.538876124113076</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.0149261917510183</v>
+        <v>-0.015846882970267</v>
       </c>
     </row>
     <row r="16">
@@ -8433,10 +8433,10 @@
         <v>0.591605525530161</v>
       </c>
       <c r="D16" t="n">
-        <v>0.574504418651013</v>
+        <v>0.573580990444202</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0171011068791482</v>
+        <v>-0.0180245350859591</v>
       </c>
     </row>
     <row r="17">
@@ -8450,10 +8450,10 @@
         <v>0.554723007083343</v>
       </c>
       <c r="D17" t="n">
-        <v>0.581295341663322</v>
+        <v>0.580604621671912</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0265723345799795</v>
+        <v>0.0258816145885689</v>
       </c>
     </row>
     <row r="18">
@@ -8467,10 +8467,10 @@
         <v>0.591605525530161</v>
       </c>
       <c r="D18" t="n">
-        <v>0.620252009117291</v>
+        <v>0.619608861337528</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0286464835871295</v>
+        <v>0.0280033358073667</v>
       </c>
     </row>
     <row r="19">
@@ -8656,25 +8656,25 @@
         <v>-542.934369809947</v>
       </c>
       <c r="D7" t="n">
-        <v>-541.186839094373</v>
+        <v>-540.74594176429</v>
       </c>
       <c r="E7" t="n">
         <v>10.1634780492893</v>
       </c>
       <c r="F7" t="n">
-        <v>10.231704661376</v>
+        <v>10.2666709427895</v>
       </c>
       <c r="G7" t="n">
-        <v>4.93282580759551</v>
+        <v>5.16018900043502</v>
       </c>
       <c r="H7" t="n">
         <v>-0.0187195333624707</v>
       </c>
       <c r="I7" t="n">
-        <v>-0.0189060485626329</v>
+        <v>-0.0189861266629066</v>
       </c>
       <c r="J7" t="n">
-        <v>-0.000186515200162194</v>
+        <v>-0.00026659330043587</v>
       </c>
     </row>
     <row r="8">
@@ -8688,25 +8688,25 @@
         <v>388.015540628305</v>
       </c>
       <c r="D8" t="n">
-        <v>389.404928707417</v>
+        <v>390.270688126179</v>
       </c>
       <c r="E8" t="n">
         <v>-22.1320199327549</v>
       </c>
       <c r="F8" t="n">
-        <v>-22.1071293786188</v>
+        <v>-22.088326290751</v>
       </c>
       <c r="G8" t="n">
-        <v>3.73711427320941</v>
+        <v>4.44061111078881</v>
       </c>
       <c r="H8" t="n">
         <v>-0.0570390038938054</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.056771570539697</v>
+        <v>-0.0565974513658827</v>
       </c>
       <c r="J8" t="n">
-        <v>0.000267433354108421</v>
+        <v>0.00044155252792269</v>
       </c>
     </row>
     <row r="9">
@@ -8720,25 +8720,25 @@
         <v>561.153333258383</v>
       </c>
       <c r="D9" t="n">
-        <v>563.521051089097</v>
+        <v>564.683335096178</v>
       </c>
       <c r="E9" t="n">
         <v>-28.3209534736833</v>
       </c>
       <c r="F9" t="n">
-        <v>-28.1994105760795</v>
+        <v>-28.0997517441893</v>
       </c>
       <c r="G9" t="n">
-        <v>4.96649151321292</v>
+        <v>5.93581188577805</v>
       </c>
       <c r="H9" t="n">
         <v>-0.0504691887139569</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.0500414501314183</v>
+        <v>-0.0497619639145244</v>
       </c>
       <c r="J9" t="n">
-        <v>0.000427738582538591</v>
+        <v>0.000707224799432533</v>
       </c>
     </row>
     <row r="10">
@@ -8752,25 +8752,25 @@
         <v>820.169437223817</v>
       </c>
       <c r="D10" t="n">
-        <v>825.403189936321</v>
+        <v>827.191729845625</v>
       </c>
       <c r="E10" t="n">
         <v>-11.9244988869571</v>
       </c>
       <c r="F10" t="n">
-        <v>-11.4781676929823</v>
+        <v>-11.2310971724855</v>
       </c>
       <c r="G10" t="n">
-        <v>8.23800074739656</v>
+        <v>9.80103293915134</v>
       </c>
       <c r="H10" t="n">
         <v>-0.0145390675947646</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.0139061343994416</v>
+        <v>-0.0135773808746631</v>
       </c>
       <c r="J10" t="n">
-        <v>0.000632933195322982</v>
+        <v>0.000961686720101449</v>
       </c>
     </row>
     <row r="11">
@@ -8784,25 +8784,25 @@
         <v>1092.09465240244</v>
       </c>
       <c r="D11" t="n">
-        <v>1099.96809318682</v>
+        <v>1102.63940626043</v>
       </c>
       <c r="E11" t="n">
         <v>25.8751535659036</v>
       </c>
       <c r="F11" t="n">
-        <v>26.7877728247676</v>
+        <v>27.1935558299538</v>
       </c>
       <c r="G11" t="n">
-        <v>12.0742934892872</v>
+        <v>14.4406703464036</v>
       </c>
       <c r="H11" t="n">
         <v>0.0236931418984446</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0243532271442149</v>
+        <v>0.0246622383306434</v>
       </c>
       <c r="J11" t="n">
-        <v>0.00066008524577028</v>
+        <v>0.000969096432198703</v>
       </c>
     </row>
     <row r="12">
@@ -8816,25 +8816,25 @@
         <v>1431.3633583382</v>
       </c>
       <c r="D12" t="n">
-        <v>1444.93248117113</v>
+        <v>1447.98085444721</v>
       </c>
       <c r="E12" t="n">
         <v>69.7612385491509</v>
       </c>
       <c r="F12" t="n">
-        <v>71.5964955593766</v>
+        <v>72.0208322509512</v>
       </c>
       <c r="G12" t="n">
-        <v>16.9469317494115</v>
+        <v>19.7291984804921</v>
       </c>
       <c r="H12" t="n">
         <v>0.0487376165826566</v>
       </c>
       <c r="I12" t="n">
-        <v>0.0495500630599342</v>
+        <v>0.0497388014694754</v>
       </c>
       <c r="J12" t="n">
-        <v>0.000812446477277552</v>
+        <v>0.00100118488681884</v>
       </c>
     </row>
     <row r="13">
@@ -8848,25 +8848,25 @@
         <v>1878.29534636384</v>
       </c>
       <c r="D13" t="n">
-        <v>1896.09950679296</v>
+        <v>1900.44020918619</v>
       </c>
       <c r="E13" t="n">
         <v>121.053987882839</v>
       </c>
       <c r="F13" t="n">
-        <v>123.964657638373</v>
+        <v>124.669209569249</v>
       </c>
       <c r="G13" t="n">
-        <v>21.3771193190147</v>
+        <v>25.4107572160766</v>
       </c>
       <c r="H13" t="n">
         <v>0.0644488568409571</v>
       </c>
       <c r="I13" t="n">
-        <v>0.0653787721552891</v>
+        <v>0.0656001746156671</v>
       </c>
       <c r="J13" t="n">
-        <v>0.00092991531433205</v>
+        <v>0.00115131777471005</v>
       </c>
     </row>
     <row r="14">
@@ -8880,25 +8880,25 @@
         <v>2601.56180865961</v>
       </c>
       <c r="D14" t="n">
-        <v>2629.46108682173</v>
+        <v>2634.77964641</v>
       </c>
       <c r="E14" t="n">
         <v>208.271689492574</v>
       </c>
       <c r="F14" t="n">
-        <v>212.527529826021</v>
+        <v>213.338761089669</v>
       </c>
       <c r="G14" t="n">
-        <v>32.8120623196846</v>
+        <v>37.7228906344572</v>
       </c>
       <c r="H14" t="n">
         <v>0.0800564064245242</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0808255086531462</v>
+        <v>0.0809702478840506</v>
       </c>
       <c r="J14" t="n">
-        <v>0.000769102228622018</v>
+        <v>0.000913841459526429</v>
       </c>
     </row>
     <row r="15">
@@ -8912,25 +8912,25 @@
         <v>3791.68208048503</v>
       </c>
       <c r="D15" t="n">
-        <v>3849.88434871667</v>
+        <v>3855.70317566834</v>
       </c>
       <c r="E15" t="n">
         <v>402.378381436465</v>
       </c>
       <c r="F15" t="n">
-        <v>414.299876266921</v>
+        <v>415.535123456967</v>
       </c>
       <c r="G15" t="n">
-        <v>54.6280517434375</v>
+        <v>60.5267220778903</v>
       </c>
       <c r="H15" t="n">
         <v>0.106121339525647</v>
       </c>
       <c r="I15" t="n">
-        <v>0.107613590108239</v>
+        <v>0.107771554117347</v>
       </c>
       <c r="J15" t="n">
-        <v>0.00149225058259175</v>
+        <v>0.00165021459169955</v>
       </c>
     </row>
     <row r="16">
@@ -8944,25 +8944,25 @@
         <v>11740.8308088609</v>
       </c>
       <c r="D16" t="n">
-        <v>11967.6526776531</v>
+        <v>11982.3746163151</v>
       </c>
       <c r="E16" t="n">
         <v>2177.01364224858</v>
       </c>
       <c r="F16" t="n">
-        <v>2232.0334604589</v>
+        <v>2237.06661735816</v>
       </c>
       <c r="G16" t="n">
-        <v>244.22959702204</v>
+        <v>257.585174594909</v>
       </c>
       <c r="H16" t="n">
         <v>0.185422452438849</v>
       </c>
       <c r="I16" t="n">
-        <v>0.186505534592153</v>
+        <v>0.186696434470692</v>
       </c>
       <c r="J16" t="n">
-        <v>0.00108308215330408</v>
+        <v>0.00127398203184365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Paper exhibits: pin A1/A2 to the publication data vintage; revise Fig 2 title
The appendix charts (A1 GDP growth, A2 labor share) pulled live FRED
data, so the v1.0.1 re-run picked up 2026 Q2 and revisions released after
publication: A2's 2026 point moved from 53.67% to 53.19%. Fetch every
series from ALFRED at the 2026-07-09 vintage (the v1.0.0 build date;
identical to the 2026-07-20 release-day vintage). The A1 and A2 historical
series now reproduce the published v1.0.0 workbook exactly.

A2's latest year is a partial-year average; flag it in a new Coverage
column and label it "2026 YTD" on the PNG. Notes lines state the vintage.

Figure 2 caption -> "Capital and corporate revenue gains drive the
increase; labor revenue falls mainly under slow adoption" (sheet + Data
TOC). Erratum note updated for the new title and the A2 history.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/figures/2030/paper_figure_data_2030.xlsx
+++ b/results/figures/2030/paper_figure_data_2030.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="241">
   <si>
     <t xml:space="preserve">AI-Fiscal — paper exhibits (FY 2030)</t>
   </si>
@@ -68,7 +68,7 @@
     <t xml:space="preserve">F2</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure 2. Capital and corporate revenue increases offset labor revenue losses in most scenarios</t>
+    <t xml:space="preserve">Figure 2. Capital and corporate revenue gains drive the increase; labor revenue falls mainly under slow adoption</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue change decomposed by type of income</t>
@@ -527,7 +527,7 @@
     <t xml:space="preserve">Subtitle: GDP growth (5-yr annualized, log). CBO projection 2026 onward.</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: Real GDP from FRED GDPC1 (Bil. Chn. 2017$). 5-yr annualized log growth; projection extends GDP with the CBO baseline path. Reference lines = AI scenario GDP CAGRs.</t>
+    <t xml:space="preserve">Notes: Real GDP from FRED GDPC1 (Bil. Chn. 2017$). 5-yr annualized log growth; projection extends GDP with the CBO baseline path. Reference lines = AI scenario GDP CAGRs. Data vintage: 2026-07-09 (ALFRED).</t>
   </si>
   <si>
     <t xml:space="preserve">Source: BEA/BLS via FRED (GDPC1), CBO February 2026 baseline, NBER recessions; The Budget Lab at Yale.</t>
@@ -554,13 +554,22 @@
     <t xml:space="preserve">Subtitle: Labor share of income (nonfarm business, percent)</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: Labor share from FRED PRS85006173 (BLS NFB labor share, index 2017=100), rescaled to percent at the 2017 level. Reference lines = AI scenario 2030 labor shares.</t>
+    <t xml:space="preserve">Notes: Labor share from FRED PRS85006173 (BLS NFB labor share, index 2017=100), rescaled to percent at the 2017 level. Annual averages of quarterly data; the latest year is a year-to-date average of the quarters available at publication (see Coverage). Reference lines = AI scenario 2030 labor shares. Data vintage: 2026-07-09 (ALFRED).</t>
   </si>
   <si>
     <t xml:space="preserve">Source: BLS via FRED (PRS85006173), NBER recessions; The Budget Lab at Yale.</t>
   </si>
   <si>
     <t xml:space="preserve">Labor Share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coverage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Year to date (Q1)</t>
   </si>
   <si>
     <t xml:space="preserve">Subtitle: Change in federal revenue (y-axis) plotted against pre-tax income growth (x-axis), FY 2030, Billions USD</t>
@@ -2571,7 +2580,7 @@
         <v>2021</v>
       </c>
       <c r="B76" t="n">
-        <v>0.0237573082522044</v>
+        <v>0.0235382702054906</v>
       </c>
       <c r="C76"/>
       <c r="D76" t="n">
@@ -2589,7 +2598,7 @@
         <v>2022</v>
       </c>
       <c r="B77" t="n">
-        <v>0.0237025923488549</v>
+        <v>0.0236682162326723</v>
       </c>
       <c r="C77"/>
       <c r="D77" t="n">
@@ -2607,7 +2616,7 @@
         <v>2023</v>
       </c>
       <c r="B78" t="n">
-        <v>0.0236094464296709</v>
+        <v>0.0236057828903334</v>
       </c>
       <c r="C78"/>
       <c r="D78" t="n">
@@ -2625,7 +2634,7 @@
         <v>2024</v>
       </c>
       <c r="B79" t="n">
-        <v>0.0243254433617899</v>
+        <v>0.0240135318044857</v>
       </c>
       <c r="C79"/>
       <c r="D79" t="n">
@@ -2643,10 +2652,10 @@
         <v>2025</v>
       </c>
       <c r="B80" t="n">
-        <v>0.0331663413820539</v>
+        <v>0.0323891425079967</v>
       </c>
       <c r="C80" t="n">
-        <v>0.0331663413820539</v>
+        <v>0.0323891425079967</v>
       </c>
       <c r="D80" t="n">
         <v>0.02</v>
@@ -2664,7 +2673,7 @@
       </c>
       <c r="B81"/>
       <c r="C81" t="n">
-        <v>0.0253591906876665</v>
+        <v>0.024801029860323</v>
       </c>
       <c r="D81" t="n">
         <v>0.02</v>
@@ -2682,7 +2691,7 @@
       </c>
       <c r="B82"/>
       <c r="C82" t="n">
-        <v>0.0241260705015787</v>
+        <v>0.0233832477437041</v>
       </c>
       <c r="D82" t="n">
         <v>0.02</v>
@@ -2700,7 +2709,7 @@
       </c>
       <c r="B83"/>
       <c r="C83" t="n">
-        <v>0.0219405014030229</v>
+        <v>0.0211669660683029</v>
       </c>
       <c r="D83" t="n">
         <v>0.02</v>
@@ -2718,7 +2727,7 @@
       </c>
       <c r="B84"/>
       <c r="C84" t="n">
-        <v>0.0196904585479317</v>
+        <v>0.0192251712311784</v>
       </c>
       <c r="D84" t="n">
         <v>0.02</v>
@@ -2736,7 +2745,7 @@
       </c>
       <c r="B85"/>
       <c r="C85" t="n">
-        <v>0.0186242328589675</v>
+        <v>0.0186242328589671</v>
       </c>
       <c r="D85" t="n">
         <v>0.02</v>
@@ -2790,7 +2799,7 @@
       </c>
       <c r="B88"/>
       <c r="C88" t="n">
-        <v>0.0178399181283307</v>
+        <v>0.0178399181283311</v>
       </c>
       <c r="D88" t="n">
         <v>0.02</v>
@@ -2808,7 +2817,7 @@
       </c>
       <c r="B89"/>
       <c r="C89" t="n">
-        <v>0.0178399181283307</v>
+        <v>0.0178399181283311</v>
       </c>
       <c r="D89" t="n">
         <v>0.02</v>
@@ -2826,7 +2835,7 @@
       </c>
       <c r="B90"/>
       <c r="C90" t="n">
-        <v>0.0178399181283307</v>
+        <v>0.0178399181283311</v>
       </c>
       <c r="D90" t="n">
         <v>0.02</v>
@@ -2868,10 +2877,11 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="19.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="13.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="19.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="13.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="17.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2902,12 +2912,15 @@
         <v>178</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2918,13 +2931,16 @@
       <c r="B7" t="n">
         <v>0.651496080117596</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D7" t="n">
         <v>0.55</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>0.54</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -2935,13 +2951,16 @@
       <c r="B8" t="n">
         <v>0.647027064188074</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D8" t="n">
         <v>0.55</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>0.54</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -2952,13 +2971,16 @@
       <c r="B9" t="n">
         <v>0.640371563853084</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="s">
+        <v>180</v>
+      </c>
+      <c r="D9" t="n">
         <v>0.55</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>0.54</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -2969,13 +2991,16 @@
       <c r="B10" t="n">
         <v>0.629146763097107</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="s">
+        <v>180</v>
+      </c>
+      <c r="D10" t="n">
         <v>0.55</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>0.54</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -2986,13 +3011,16 @@
       <c r="B11" t="n">
         <v>0.625696129116126</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="s">
+        <v>180</v>
+      </c>
+      <c r="D11" t="n">
         <v>0.55</v>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>0.54</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3003,13 +3031,16 @@
       <c r="B12" t="n">
         <v>0.634798006059818</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D12" t="n">
         <v>0.55</v>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>0.54</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3020,13 +3051,16 @@
       <c r="B13" t="n">
         <v>0.641966228513145</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" t="s">
+        <v>180</v>
+      </c>
+      <c r="D13" t="n">
         <v>0.55</v>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>0.54</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3037,13 +3071,16 @@
       <c r="B14" t="n">
         <v>0.643791123766287</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" t="s">
+        <v>180</v>
+      </c>
+      <c r="D14" t="n">
         <v>0.55</v>
       </c>
-      <c r="D14" t="n">
+      <c r="E14" t="n">
         <v>0.54</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3054,13 +3091,16 @@
       <c r="B15" t="n">
         <v>0.628735737927862</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D15" t="n">
         <v>0.55</v>
       </c>
-      <c r="D15" t="n">
+      <c r="E15" t="n">
         <v>0.54</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3071,13 +3111,16 @@
       <c r="B16" t="n">
         <v>0.648065220543384</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" t="s">
+        <v>180</v>
+      </c>
+      <c r="D16" t="n">
         <v>0.55</v>
       </c>
-      <c r="D16" t="n">
+      <c r="E16" t="n">
         <v>0.54</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3088,13 +3131,16 @@
       <c r="B17" t="n">
         <v>0.647753067407978</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" t="s">
+        <v>180</v>
+      </c>
+      <c r="D17" t="n">
         <v>0.55</v>
       </c>
-      <c r="D17" t="n">
+      <c r="E17" t="n">
         <v>0.54</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3105,13 +3151,16 @@
       <c r="B18" t="n">
         <v>0.648798286051418</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" t="s">
+        <v>180</v>
+      </c>
+      <c r="D18" t="n">
         <v>0.55</v>
       </c>
-      <c r="D18" t="n">
+      <c r="E18" t="n">
         <v>0.54</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3122,13 +3171,16 @@
       <c r="B19" t="n">
         <v>0.640543883683489</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" t="s">
+        <v>180</v>
+      </c>
+      <c r="D19" t="n">
         <v>0.55</v>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
         <v>0.54</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3139,13 +3191,16 @@
       <c r="B20" t="n">
         <v>0.652715031049068</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" t="s">
+        <v>180</v>
+      </c>
+      <c r="D20" t="n">
         <v>0.55</v>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>0.54</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3156,13 +3211,16 @@
       <c r="B21" t="n">
         <v>0.648073695289141</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" t="s">
+        <v>180</v>
+      </c>
+      <c r="D21" t="n">
         <v>0.55</v>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>0.54</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3173,13 +3231,16 @@
       <c r="B22" t="n">
         <v>0.638961931142066</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" t="s">
+        <v>180</v>
+      </c>
+      <c r="D22" t="n">
         <v>0.55</v>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>0.54</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3190,13 +3251,16 @@
       <c r="B23" t="n">
         <v>0.633975955721328</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" t="s">
+        <v>180</v>
+      </c>
+      <c r="D23" t="n">
         <v>0.55</v>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>0.54</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3207,13 +3271,16 @@
       <c r="B24" t="n">
         <v>0.627180622081338</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" t="s">
+        <v>180</v>
+      </c>
+      <c r="D24" t="n">
         <v>0.55</v>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
         <v>0.54</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3224,13 +3291,16 @@
       <c r="B25" t="n">
         <v>0.620091497255082</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" t="s">
+        <v>180</v>
+      </c>
+      <c r="D25" t="n">
         <v>0.55</v>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
         <v>0.54</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3241,13 +3311,16 @@
       <c r="B26" t="n">
         <v>0.619748270051898</v>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" t="s">
+        <v>180</v>
+      </c>
+      <c r="D26" t="n">
         <v>0.55</v>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
         <v>0.54</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3258,13 +3331,16 @@
       <c r="B27" t="n">
         <v>0.624398080557583</v>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" t="s">
+        <v>180</v>
+      </c>
+      <c r="D27" t="n">
         <v>0.55</v>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
         <v>0.54</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3275,13 +3351,16 @@
       <c r="B28" t="n">
         <v>0.624547801065968</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" t="s">
+        <v>180</v>
+      </c>
+      <c r="D28" t="n">
         <v>0.55</v>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
         <v>0.54</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3292,13 +3371,16 @@
       <c r="B29" t="n">
         <v>0.637504274871754</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" t="s">
+        <v>180</v>
+      </c>
+      <c r="D29" t="n">
         <v>0.55</v>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="n">
         <v>0.54</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3309,13 +3391,16 @@
       <c r="B30" t="n">
         <v>0.643832085037449</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" t="s">
+        <v>180</v>
+      </c>
+      <c r="D30" t="n">
         <v>0.55</v>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
         <v>0.54</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3326,13 +3411,16 @@
       <c r="B31" t="n">
         <v>0.630288028859134</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" t="s">
+        <v>180</v>
+      </c>
+      <c r="D31" t="n">
         <v>0.55</v>
       </c>
-      <c r="D31" t="n">
+      <c r="E31" t="n">
         <v>0.54</v>
       </c>
-      <c r="E31" t="n">
+      <c r="F31" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3343,13 +3431,16 @@
       <c r="B32" t="n">
         <v>0.629597337079888</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" t="s">
+        <v>180</v>
+      </c>
+      <c r="D32" t="n">
         <v>0.55</v>
       </c>
-      <c r="D32" t="n">
+      <c r="E32" t="n">
         <v>0.54</v>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3360,13 +3451,16 @@
       <c r="B33" t="n">
         <v>0.634768344449667</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" t="s">
+        <v>180</v>
+      </c>
+      <c r="D33" t="n">
         <v>0.55</v>
       </c>
-      <c r="D33" t="n">
+      <c r="E33" t="n">
         <v>0.54</v>
       </c>
-      <c r="E33" t="n">
+      <c r="F33" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3377,13 +3471,16 @@
       <c r="B34" t="n">
         <v>0.640108846734598</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" t="s">
+        <v>180</v>
+      </c>
+      <c r="D34" t="n">
         <v>0.55</v>
       </c>
-      <c r="D34" t="n">
+      <c r="E34" t="n">
         <v>0.54</v>
       </c>
-      <c r="E34" t="n">
+      <c r="F34" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3394,13 +3491,16 @@
       <c r="B35" t="n">
         <v>0.622261032169035</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" t="s">
+        <v>180</v>
+      </c>
+      <c r="D35" t="n">
         <v>0.55</v>
       </c>
-      <c r="D35" t="n">
+      <c r="E35" t="n">
         <v>0.54</v>
       </c>
-      <c r="E35" t="n">
+      <c r="F35" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3411,13 +3511,16 @@
       <c r="B36" t="n">
         <v>0.614447316580503</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" t="s">
+        <v>180</v>
+      </c>
+      <c r="D36" t="n">
         <v>0.55</v>
       </c>
-      <c r="D36" t="n">
+      <c r="E36" t="n">
         <v>0.54</v>
       </c>
-      <c r="E36" t="n">
+      <c r="F36" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3428,13 +3531,16 @@
       <c r="B37" t="n">
         <v>0.615265129546114</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" t="s">
+        <v>180</v>
+      </c>
+      <c r="D37" t="n">
         <v>0.55</v>
       </c>
-      <c r="D37" t="n">
+      <c r="E37" t="n">
         <v>0.54</v>
       </c>
-      <c r="E37" t="n">
+      <c r="F37" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3445,13 +3551,16 @@
       <c r="B38" t="n">
         <v>0.618594292171235</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" t="s">
+        <v>180</v>
+      </c>
+      <c r="D38" t="n">
         <v>0.55</v>
       </c>
-      <c r="D38" t="n">
+      <c r="E38" t="n">
         <v>0.54</v>
       </c>
-      <c r="E38" t="n">
+      <c r="F38" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3462,13 +3571,16 @@
       <c r="B39" t="n">
         <v>0.626265349539514</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C39" t="s">
+        <v>180</v>
+      </c>
+      <c r="D39" t="n">
         <v>0.55</v>
       </c>
-      <c r="D39" t="n">
+      <c r="E39" t="n">
         <v>0.54</v>
       </c>
-      <c r="E39" t="n">
+      <c r="F39" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3479,13 +3591,16 @@
       <c r="B40" t="n">
         <v>0.633559280721578</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C40" t="s">
+        <v>180</v>
+      </c>
+      <c r="D40" t="n">
         <v>0.55</v>
       </c>
-      <c r="D40" t="n">
+      <c r="E40" t="n">
         <v>0.54</v>
       </c>
-      <c r="E40" t="n">
+      <c r="F40" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3496,13 +3611,16 @@
       <c r="B41" t="n">
         <v>0.624471528354149</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" t="s">
+        <v>180</v>
+      </c>
+      <c r="D41" t="n">
         <v>0.55</v>
       </c>
-      <c r="D41" t="n">
+      <c r="E41" t="n">
         <v>0.54</v>
       </c>
-      <c r="E41" t="n">
+      <c r="F41" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3513,13 +3631,16 @@
       <c r="B42" t="n">
         <v>0.636333347499575</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" t="s">
+        <v>180</v>
+      </c>
+      <c r="D42" t="n">
         <v>0.55</v>
       </c>
-      <c r="D42" t="n">
+      <c r="E42" t="n">
         <v>0.54</v>
       </c>
-      <c r="E42" t="n">
+      <c r="F42" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3530,13 +3651,16 @@
       <c r="B43" t="n">
         <v>0.617258107256782</v>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" t="s">
+        <v>180</v>
+      </c>
+      <c r="D43" t="n">
         <v>0.55</v>
       </c>
-      <c r="D43" t="n">
+      <c r="E43" t="n">
         <v>0.54</v>
       </c>
-      <c r="E43" t="n">
+      <c r="F43" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3547,13 +3671,16 @@
       <c r="B44" t="n">
         <v>0.612554623361299</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" t="s">
+        <v>180</v>
+      </c>
+      <c r="D44" t="n">
         <v>0.55</v>
       </c>
-      <c r="D44" t="n">
+      <c r="E44" t="n">
         <v>0.54</v>
       </c>
-      <c r="E44" t="n">
+      <c r="F44" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3564,13 +3691,16 @@
       <c r="B45" t="n">
         <v>0.612718468445947</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C45" t="s">
+        <v>180</v>
+      </c>
+      <c r="D45" t="n">
         <v>0.55</v>
       </c>
-      <c r="D45" t="n">
+      <c r="E45" t="n">
         <v>0.54</v>
       </c>
-      <c r="E45" t="n">
+      <c r="F45" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3581,13 +3711,16 @@
       <c r="B46" t="n">
         <v>0.620470035898923</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C46" t="s">
+        <v>180</v>
+      </c>
+      <c r="D46" t="n">
         <v>0.55</v>
       </c>
-      <c r="D46" t="n">
+      <c r="E46" t="n">
         <v>0.54</v>
       </c>
-      <c r="E46" t="n">
+      <c r="F46" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3598,13 +3731,16 @@
       <c r="B47" t="n">
         <v>0.628612854114377</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C47" t="s">
+        <v>180</v>
+      </c>
+      <c r="D47" t="n">
         <v>0.55</v>
       </c>
-      <c r="D47" t="n">
+      <c r="E47" t="n">
         <v>0.54</v>
       </c>
-      <c r="E47" t="n">
+      <c r="F47" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3615,13 +3751,16 @@
       <c r="B48" t="n">
         <v>0.630908097757067</v>
       </c>
-      <c r="C48" t="n">
+      <c r="C48" t="s">
+        <v>180</v>
+      </c>
+      <c r="D48" t="n">
         <v>0.55</v>
       </c>
-      <c r="D48" t="n">
+      <c r="E48" t="n">
         <v>0.54</v>
       </c>
-      <c r="E48" t="n">
+      <c r="F48" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3632,13 +3771,16 @@
       <c r="B49" t="n">
         <v>0.620794901152965</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C49" t="s">
+        <v>180</v>
+      </c>
+      <c r="D49" t="n">
         <v>0.55</v>
       </c>
-      <c r="D49" t="n">
+      <c r="E49" t="n">
         <v>0.54</v>
       </c>
-      <c r="E49" t="n">
+      <c r="F49" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3649,13 +3791,16 @@
       <c r="B50" t="n">
         <v>0.625567595472136</v>
       </c>
-      <c r="C50" t="n">
+      <c r="C50" t="s">
+        <v>180</v>
+      </c>
+      <c r="D50" t="n">
         <v>0.55</v>
       </c>
-      <c r="D50" t="n">
+      <c r="E50" t="n">
         <v>0.54</v>
       </c>
-      <c r="E50" t="n">
+      <c r="F50" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3666,13 +3811,16 @@
       <c r="B51" t="n">
         <v>0.625273804285871</v>
       </c>
-      <c r="C51" t="n">
+      <c r="C51" t="s">
+        <v>180</v>
+      </c>
+      <c r="D51" t="n">
         <v>0.55</v>
       </c>
-      <c r="D51" t="n">
+      <c r="E51" t="n">
         <v>0.54</v>
       </c>
-      <c r="E51" t="n">
+      <c r="F51" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3683,13 +3831,16 @@
       <c r="B52" t="n">
         <v>0.625246967590972</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C52" t="s">
+        <v>180</v>
+      </c>
+      <c r="D52" t="n">
         <v>0.55</v>
       </c>
-      <c r="D52" t="n">
+      <c r="E52" t="n">
         <v>0.54</v>
       </c>
-      <c r="E52" t="n">
+      <c r="F52" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3700,13 +3851,16 @@
       <c r="B53" t="n">
         <v>0.617721393358199</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C53" t="s">
+        <v>180</v>
+      </c>
+      <c r="D53" t="n">
         <v>0.55</v>
       </c>
-      <c r="D53" t="n">
+      <c r="E53" t="n">
         <v>0.54</v>
       </c>
-      <c r="E53" t="n">
+      <c r="F53" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3717,13 +3871,16 @@
       <c r="B54" t="n">
         <v>0.608232503024909</v>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" t="s">
+        <v>180</v>
+      </c>
+      <c r="D54" t="n">
         <v>0.55</v>
       </c>
-      <c r="D54" t="n">
+      <c r="E54" t="n">
         <v>0.54</v>
       </c>
-      <c r="E54" t="n">
+      <c r="F54" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3734,13 +3891,16 @@
       <c r="B55" t="n">
         <v>0.605877936161915</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C55" t="s">
+        <v>180</v>
+      </c>
+      <c r="D55" t="n">
         <v>0.55</v>
       </c>
-      <c r="D55" t="n">
+      <c r="E55" t="n">
         <v>0.54</v>
       </c>
-      <c r="E55" t="n">
+      <c r="F55" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3751,13 +3911,16 @@
       <c r="B56" t="n">
         <v>0.605537533873984</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C56" t="s">
+        <v>180</v>
+      </c>
+      <c r="D56" t="n">
         <v>0.55</v>
       </c>
-      <c r="D56" t="n">
+      <c r="E56" t="n">
         <v>0.54</v>
       </c>
-      <c r="E56" t="n">
+      <c r="F56" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3768,13 +3931,16 @@
       <c r="B57" t="n">
         <v>0.60662230133096</v>
       </c>
-      <c r="C57" t="n">
+      <c r="C57" t="s">
+        <v>180</v>
+      </c>
+      <c r="D57" t="n">
         <v>0.55</v>
       </c>
-      <c r="D57" t="n">
+      <c r="E57" t="n">
         <v>0.54</v>
       </c>
-      <c r="E57" t="n">
+      <c r="F57" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3785,13 +3951,16 @@
       <c r="B58" t="n">
         <v>0.618667739967801</v>
       </c>
-      <c r="C58" t="n">
+      <c r="C58" t="s">
+        <v>180</v>
+      </c>
+      <c r="D58" t="n">
         <v>0.55</v>
       </c>
-      <c r="D58" t="n">
+      <c r="E58" t="n">
         <v>0.54</v>
       </c>
-      <c r="E58" t="n">
+      <c r="F58" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3802,13 +3971,16 @@
       <c r="B59" t="n">
         <v>0.618669152425427</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C59" t="s">
+        <v>180</v>
+      </c>
+      <c r="D59" t="n">
         <v>0.55</v>
       </c>
-      <c r="D59" t="n">
+      <c r="E59" t="n">
         <v>0.54</v>
       </c>
-      <c r="E59" t="n">
+      <c r="F59" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3819,13 +3991,16 @@
       <c r="B60" t="n">
         <v>0.630625606231813</v>
       </c>
-      <c r="C60" t="n">
+      <c r="C60" t="s">
+        <v>180</v>
+      </c>
+      <c r="D60" t="n">
         <v>0.55</v>
       </c>
-      <c r="D60" t="n">
+      <c r="E60" t="n">
         <v>0.54</v>
       </c>
-      <c r="E60" t="n">
+      <c r="F60" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3836,13 +4011,16 @@
       <c r="B61" t="n">
         <v>0.631213188604342</v>
       </c>
-      <c r="C61" t="n">
+      <c r="C61" t="s">
+        <v>180</v>
+      </c>
+      <c r="D61" t="n">
         <v>0.55</v>
       </c>
-      <c r="D61" t="n">
+      <c r="E61" t="n">
         <v>0.54</v>
       </c>
-      <c r="E61" t="n">
+      <c r="F61" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3853,13 +4031,16 @@
       <c r="B62" t="n">
         <v>0.614056065818025</v>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" t="s">
+        <v>180</v>
+      </c>
+      <c r="D62" t="n">
         <v>0.55</v>
       </c>
-      <c r="D62" t="n">
+      <c r="E62" t="n">
         <v>0.54</v>
       </c>
-      <c r="E62" t="n">
+      <c r="F62" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3870,13 +4051,16 @@
       <c r="B63" t="n">
         <v>0.605999407517774</v>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" t="s">
+        <v>180</v>
+      </c>
+      <c r="D63" t="n">
         <v>0.55</v>
       </c>
-      <c r="D63" t="n">
+      <c r="E63" t="n">
         <v>0.54</v>
       </c>
-      <c r="E63" t="n">
+      <c r="F63" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3887,13 +4071,16 @@
       <c r="B64" t="n">
         <v>0.601185751927442</v>
       </c>
-      <c r="C64" t="n">
+      <c r="C64" t="s">
+        <v>180</v>
+      </c>
+      <c r="D64" t="n">
         <v>0.55</v>
       </c>
-      <c r="D64" t="n">
+      <c r="E64" t="n">
         <v>0.54</v>
       </c>
-      <c r="E64" t="n">
+      <c r="F64" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3904,13 +4091,16 @@
       <c r="B65" t="n">
         <v>0.589972250832475</v>
       </c>
-      <c r="C65" t="n">
+      <c r="C65" t="s">
+        <v>180</v>
+      </c>
+      <c r="D65" t="n">
         <v>0.55</v>
       </c>
-      <c r="D65" t="n">
+      <c r="E65" t="n">
         <v>0.54</v>
       </c>
-      <c r="E65" t="n">
+      <c r="F65" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3921,13 +4111,16 @@
       <c r="B66" t="n">
         <v>0.589434104476866</v>
       </c>
-      <c r="C66" t="n">
+      <c r="C66" t="s">
+        <v>180</v>
+      </c>
+      <c r="D66" t="n">
         <v>0.55</v>
       </c>
-      <c r="D66" t="n">
+      <c r="E66" t="n">
         <v>0.54</v>
       </c>
-      <c r="E66" t="n">
+      <c r="F66" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3938,13 +4131,16 @@
       <c r="B67" t="n">
         <v>0.592462413627591</v>
       </c>
-      <c r="C67" t="n">
+      <c r="C67" t="s">
+        <v>180</v>
+      </c>
+      <c r="D67" t="n">
         <v>0.55</v>
       </c>
-      <c r="D67" t="n">
+      <c r="E67" t="n">
         <v>0.54</v>
       </c>
-      <c r="E67" t="n">
+      <c r="F67" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3955,13 +4151,16 @@
       <c r="B68" t="n">
         <v>0.593840972270832</v>
       </c>
-      <c r="C68" t="n">
+      <c r="C68" t="s">
+        <v>180</v>
+      </c>
+      <c r="D68" t="n">
         <v>0.55</v>
       </c>
-      <c r="D68" t="n">
+      <c r="E68" t="n">
         <v>0.54</v>
       </c>
-      <c r="E68" t="n">
+      <c r="F68" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3972,13 +4171,16 @@
       <c r="B69" t="n">
         <v>0.576309548213554</v>
       </c>
-      <c r="C69" t="n">
+      <c r="C69" t="s">
+        <v>180</v>
+      </c>
+      <c r="D69" t="n">
         <v>0.55</v>
       </c>
-      <c r="D69" t="n">
+      <c r="E69" t="n">
         <v>0.54</v>
       </c>
-      <c r="E69" t="n">
+      <c r="F69" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -3989,13 +4191,16 @@
       <c r="B70" t="n">
         <v>0.56215531034069</v>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" t="s">
+        <v>180</v>
+      </c>
+      <c r="D70" t="n">
         <v>0.55</v>
       </c>
-      <c r="D70" t="n">
+      <c r="E70" t="n">
         <v>0.54</v>
       </c>
-      <c r="E70" t="n">
+      <c r="F70" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4006,13 +4211,16 @@
       <c r="B71" t="n">
         <v>0.563409572712819</v>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" t="s">
+        <v>180</v>
+      </c>
+      <c r="D71" t="n">
         <v>0.55</v>
       </c>
-      <c r="D71" t="n">
+      <c r="E71" t="n">
         <v>0.54</v>
       </c>
-      <c r="E71" t="n">
+      <c r="F71" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4023,13 +4231,16 @@
       <c r="B72" t="n">
         <v>0.561902480425587</v>
       </c>
-      <c r="C72" t="n">
+      <c r="C72" t="s">
+        <v>180</v>
+      </c>
+      <c r="D72" t="n">
         <v>0.55</v>
       </c>
-      <c r="D72" t="n">
+      <c r="E72" t="n">
         <v>0.54</v>
       </c>
-      <c r="E72" t="n">
+      <c r="F72" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4040,13 +4251,16 @@
       <c r="B73" t="n">
         <v>0.557290806275812</v>
       </c>
-      <c r="C73" t="n">
+      <c r="C73" t="s">
+        <v>180</v>
+      </c>
+      <c r="D73" t="n">
         <v>0.55</v>
       </c>
-      <c r="D73" t="n">
+      <c r="E73" t="n">
         <v>0.54</v>
       </c>
-      <c r="E73" t="n">
+      <c r="F73" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4057,13 +4271,16 @@
       <c r="B74" t="n">
         <v>0.55778375398738</v>
       </c>
-      <c r="C74" t="n">
+      <c r="C74" t="s">
+        <v>180</v>
+      </c>
+      <c r="D74" t="n">
         <v>0.55</v>
       </c>
-      <c r="D74" t="n">
+      <c r="E74" t="n">
         <v>0.54</v>
       </c>
-      <c r="E74" t="n">
+      <c r="F74" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4074,13 +4291,16 @@
       <c r="B75" t="n">
         <v>0.563685001949942</v>
       </c>
-      <c r="C75" t="n">
+      <c r="C75" t="s">
+        <v>180</v>
+      </c>
+      <c r="D75" t="n">
         <v>0.55</v>
       </c>
-      <c r="D75" t="n">
+      <c r="E75" t="n">
         <v>0.54</v>
       </c>
-      <c r="E75" t="n">
+      <c r="F75" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4091,13 +4311,16 @@
       <c r="B76" t="n">
         <v>0.56208327500175</v>
       </c>
-      <c r="C76" t="n">
+      <c r="C76" t="s">
+        <v>180</v>
+      </c>
+      <c r="D76" t="n">
         <v>0.55</v>
       </c>
-      <c r="D76" t="n">
+      <c r="E76" t="n">
         <v>0.54</v>
       </c>
-      <c r="E76" t="n">
+      <c r="F76" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4108,13 +4331,16 @@
       <c r="B77" t="n">
         <v>0.565</v>
       </c>
-      <c r="C77" t="n">
+      <c r="C77" t="s">
+        <v>180</v>
+      </c>
+      <c r="D77" t="n">
         <v>0.55</v>
       </c>
-      <c r="D77" t="n">
+      <c r="E77" t="n">
         <v>0.54</v>
       </c>
-      <c r="E77" t="n">
+      <c r="F77" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4125,13 +4351,16 @@
       <c r="B78" t="n">
         <v>0.564057890763277</v>
       </c>
-      <c r="C78" t="n">
+      <c r="C78" t="s">
+        <v>180</v>
+      </c>
+      <c r="D78" t="n">
         <v>0.55</v>
       </c>
-      <c r="D78" t="n">
+      <c r="E78" t="n">
         <v>0.54</v>
       </c>
-      <c r="E78" t="n">
+      <c r="F78" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4142,13 +4371,16 @@
       <c r="B79" t="n">
         <v>0.565024011779647</v>
       </c>
-      <c r="C79" t="n">
+      <c r="C79" t="s">
+        <v>180</v>
+      </c>
+      <c r="D79" t="n">
         <v>0.55</v>
       </c>
-      <c r="D79" t="n">
+      <c r="E79" t="n">
         <v>0.54</v>
       </c>
-      <c r="E79" t="n">
+      <c r="F79" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4159,13 +4391,16 @@
       <c r="B80" t="n">
         <v>0.57791692499225</v>
       </c>
-      <c r="C80" t="n">
+      <c r="C80" t="s">
+        <v>180</v>
+      </c>
+      <c r="D80" t="n">
         <v>0.55</v>
       </c>
-      <c r="D80" t="n">
+      <c r="E80" t="n">
         <v>0.54</v>
       </c>
-      <c r="E80" t="n">
+      <c r="F80" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4176,13 +4411,16 @@
       <c r="B81" t="n">
         <v>0.566874331270062</v>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" t="s">
+        <v>180</v>
+      </c>
+      <c r="D81" t="n">
         <v>0.55</v>
       </c>
-      <c r="D81" t="n">
+      <c r="E81" t="n">
         <v>0.54</v>
       </c>
-      <c r="E81" t="n">
+      <c r="F81" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4193,13 +4431,16 @@
       <c r="B82" t="n">
         <v>0.55323846534604</v>
       </c>
-      <c r="C82" t="n">
+      <c r="C82" t="s">
+        <v>180</v>
+      </c>
+      <c r="D82" t="n">
         <v>0.55</v>
       </c>
-      <c r="D82" t="n">
+      <c r="E82" t="n">
         <v>0.54</v>
       </c>
-      <c r="E82" t="n">
+      <c r="F82" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4210,13 +4451,16 @@
       <c r="B83" t="n">
         <v>0.544839992300231</v>
       </c>
-      <c r="C83" t="n">
+      <c r="C83" t="s">
+        <v>180</v>
+      </c>
+      <c r="D83" t="n">
         <v>0.55</v>
       </c>
-      <c r="D83" t="n">
+      <c r="E83" t="n">
         <v>0.54</v>
       </c>
-      <c r="E83" t="n">
+      <c r="F83" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4227,13 +4471,16 @@
       <c r="B84" t="n">
         <v>0.546735510434687</v>
       </c>
-      <c r="C84" t="n">
+      <c r="C84" t="s">
+        <v>180</v>
+      </c>
+      <c r="D84" t="n">
         <v>0.55</v>
       </c>
-      <c r="D84" t="n">
+      <c r="E84" t="n">
         <v>0.54</v>
       </c>
-      <c r="E84" t="n">
+      <c r="F84" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4244,13 +4491,16 @@
       <c r="B85" t="n">
         <v>0.545660630181095</v>
       </c>
-      <c r="C85" t="n">
+      <c r="C85" t="s">
+        <v>180</v>
+      </c>
+      <c r="D85" t="n">
         <v>0.55</v>
       </c>
-      <c r="D85" t="n">
+      <c r="E85" t="n">
         <v>0.54</v>
       </c>
-      <c r="E85" t="n">
+      <c r="F85" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4259,15 +4509,18 @@
         <v>2026</v>
       </c>
       <c r="B86" t="n">
-        <v>0.53190046798596</v>
-      </c>
-      <c r="C86" t="n">
+        <v>0.53667739967801</v>
+      </c>
+      <c r="C86" t="s">
+        <v>181</v>
+      </c>
+      <c r="D86" t="n">
         <v>0.55</v>
       </c>
-      <c r="D86" t="n">
+      <c r="E86" t="n">
         <v>0.54</v>
       </c>
-      <c r="E86" t="n">
+      <c r="F86" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -4306,7 +4559,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4">
@@ -4325,40 +4578,40 @@
         <v>130</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>132</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>134</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="N6" s="3" t="s">
         <v>100</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7">
@@ -4824,7 +5077,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4">
@@ -4834,69 +5087,69 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>115</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B7"/>
       <c r="C7"/>
@@ -4942,28 +5195,28 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E8" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F8" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="G8" t="s">
         <v>88</v>
       </c>
       <c r="H8" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I8" t="n">
         <v>0.026</v>
@@ -5004,28 +5257,28 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B9" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E9" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F9" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G9" t="s">
         <v>84</v>
       </c>
       <c r="H9" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I9" t="n">
         <v>0.026</v>
@@ -5066,28 +5319,28 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B10" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C10" t="s">
         <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F10" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="G10" t="s">
         <v>90</v>
       </c>
       <c r="H10" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I10" t="n">
         <v>0.026</v>
@@ -5128,28 +5381,28 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B11" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C11" t="s">
         <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E11" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F11" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="G11" t="s">
         <v>88</v>
       </c>
       <c r="H11" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I11" t="n">
         <v>0.026</v>
@@ -5190,28 +5443,28 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B12" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C12" t="s">
         <v>50</v>
       </c>
       <c r="D12" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E12" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F12" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G12" t="s">
         <v>84</v>
       </c>
       <c r="H12" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I12" t="n">
         <v>0.026</v>
@@ -5252,28 +5505,28 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B13" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C13" t="s">
         <v>50</v>
       </c>
       <c r="D13" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E13" t="s">
+        <v>225</v>
+      </c>
+      <c r="F13" t="s">
         <v>222</v>
-      </c>
-      <c r="F13" t="s">
-        <v>219</v>
       </c>
       <c r="G13" t="s">
         <v>90</v>
       </c>
       <c r="H13" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I13" t="n">
         <v>0.026</v>
@@ -5314,28 +5567,28 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B14" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
       </c>
       <c r="D14" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E14" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F14" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="G14" t="s">
         <v>88</v>
       </c>
       <c r="H14" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I14" t="n">
         <v>0.033</v>
@@ -5376,28 +5629,28 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B15" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C15" t="s">
         <v>51</v>
       </c>
       <c r="D15" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E15" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F15" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G15" t="s">
         <v>84</v>
       </c>
       <c r="H15" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I15" t="n">
         <v>0.033</v>
@@ -5438,28 +5691,28 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B16" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E16" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F16" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="G16" t="s">
         <v>90</v>
       </c>
       <c r="H16" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I16" t="n">
         <v>0.033</v>
@@ -5500,28 +5753,28 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B17" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E17" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F17" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="G17" t="s">
         <v>88</v>
       </c>
       <c r="H17" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I17" t="n">
         <v>0.033</v>
@@ -5562,28 +5815,28 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B18" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E18" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F18" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G18" t="s">
         <v>84</v>
       </c>
       <c r="H18" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I18" t="n">
         <v>0.033</v>
@@ -5624,28 +5877,28 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B19" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E19" t="s">
+        <v>225</v>
+      </c>
+      <c r="F19" t="s">
         <v>222</v>
-      </c>
-      <c r="F19" t="s">
-        <v>219</v>
       </c>
       <c r="G19" t="s">
         <v>90</v>
       </c>
       <c r="H19" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I19" t="n">
         <v>0.033</v>
@@ -5686,28 +5939,28 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B20" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C20" t="s">
         <v>49</v>
       </c>
       <c r="D20" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E20" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F20" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="G20" t="s">
         <v>88</v>
       </c>
       <c r="H20" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I20" t="n">
         <v>0.02</v>
@@ -5748,28 +6001,28 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B21" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C21" t="s">
         <v>49</v>
       </c>
       <c r="D21" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E21" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F21" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G21" t="s">
         <v>84</v>
       </c>
       <c r="H21" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I21" t="n">
         <v>0.02</v>
@@ -5810,28 +6063,28 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B22" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C22" t="s">
         <v>49</v>
       </c>
       <c r="D22" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="E22" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F22" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="G22" t="s">
         <v>90</v>
       </c>
       <c r="H22" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I22" t="n">
         <v>0.02</v>
@@ -5872,28 +6125,28 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>238</v>
+      </c>
+      <c r="B23" t="s">
         <v>235</v>
-      </c>
-      <c r="B23" t="s">
-        <v>232</v>
       </c>
       <c r="C23" t="s">
         <v>49</v>
       </c>
       <c r="D23" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E23" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F23" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="G23" t="s">
         <v>88</v>
       </c>
       <c r="H23" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I23" t="n">
         <v>0.02</v>
@@ -5934,28 +6187,28 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B24" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C24" t="s">
         <v>49</v>
       </c>
       <c r="D24" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E24" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F24" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="G24" t="s">
         <v>84</v>
       </c>
       <c r="H24" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I24" t="n">
         <v>0.02</v>
@@ -5996,28 +6249,28 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B25" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C25" t="s">
         <v>49</v>
       </c>
       <c r="D25" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E25" t="s">
+        <v>225</v>
+      </c>
+      <c r="F25" t="s">
         <v>222</v>
-      </c>
-      <c r="F25" t="s">
-        <v>219</v>
       </c>
       <c r="G25" t="s">
         <v>90</v>
       </c>
       <c r="H25" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="I25" t="n">
         <v>0.02</v>

</xml_diff>

<commit_message>
Paper exhibits: retitle Figures 2 and 3 to match the revised article text
Updates the captions in code/paper_figure_data.R and in the generated exhibit
files (paper_figure_data CSVs for all four erratum runs, the current and v1.0.1
paper_figure_data_2030.xlsx). The v1.0.0 archive keeps the originally published titles.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/figures/2030/paper_figure_data_2030.xlsx
+++ b/results/figures/2030/paper_figure_data_2030.xlsx
@@ -68,7 +68,7 @@
     <t xml:space="preserve">F2</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure 2. Capital and corporate revenue gains drive the increase; labor revenue falls mainly under slow adoption</t>
+    <t xml:space="preserve">Figure 2. Capital and corporate revenue gains drive increased revenues</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue change decomposed by type of income</t>
@@ -77,7 +77,7 @@
     <t xml:space="preserve">F3</t>
   </si>
   <si>
-    <t xml:space="preserve">Figure 3. Revenue gains are driven by corporate and individual income tax revenue increases</t>
+    <t xml:space="preserve">Figure 3. Corporate and individual income tax revenues increase in most scenarios</t>
   </si>
   <si>
     <t xml:space="preserve">Revenue change by tax instrument</t>

</xml_diff>